<commit_message>
chore: refresh event discovery registry
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Directory" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Instructions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Source Directory" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Read me" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="User Instructions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="New White House leads" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2232,15 +2234,19 @@
           <t>daily</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:14+00:00</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>not_run</t>
+          <t>success_metadata_only</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>not_independently_checked</t>
+          <t>metadata_endpoint_reached</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2253,7 +2259,11 @@
           <t>Automated collector currently fetches recent channel upload metadata only. It does not assign event identity or verify video frames.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/gdelt0003/gdelt0003/actions/runs/38502805987</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@WhiteHouse</t>
@@ -2547,15 +2557,19 @@
           <t>daily</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:14+00:00</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>not_connected</t>
+          <t>fetch_failed</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>not_independently_checked</t>
+          <t>fetch_failed_check_run_log</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2568,7 +2582,11 @@
           <t>User-provided Explorer URL. The daily collector queries the public GDELT DOC API for article metadata only; it does not fetch article bodies or verify event facts. A live metadata response was observed during implementation; subsequent validation requests received HTTP 429, so scheduled availability and rate limits remain to be confirmed.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/gdelt0003/gdelt0003/actions/runs/38502805987</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
           <t>https://gdelt.github.io/#api=doc&amp;query=trump%20&amp;contentmode=ArtList&amp;maxrecords=250&amp;sort=DateDesc&amp;format=html&amp;timespan=1w</t>
@@ -3021,18 +3039,20 @@
   <autoFilter ref="A1:O14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3205,4 +3225,1351 @@
   <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="72" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Video ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Publisher</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Published metadata (UTC; not event time)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Upload date metadata</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Assignment status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Verified event date</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Verified event local time / timezone</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Verified location</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>President attendance duration (minutes; verified)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Speech word count (verified; language/method)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Topics (source-backed)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>First discovered UTC</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Last event verification UTC</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Page/source count (not corroboration)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>User annotation / explanation tied to source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>pvXbHQrIvTw</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 13, 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pvXbHQrIvTw</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n">
+        <v>605</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>HEWlaWY9Qcs</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 12, 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HEWlaWY9Qcs</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n">
+        <v>418</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>0ImmQBafX7Y</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Man in the Arena</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0ImmQBafX7Y</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GgnvR9UJ-Sc</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>President Trump's Second Term: Stephen Miller</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GgnvR9UJ-Sc</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>OaTi_y8_GLk</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>$5000 to Americans</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OaTi_y8_GLk</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Uf8CQeM7jHo</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Every Democrat Voted Against No Tax on Tips</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Uf8CQeM7jHo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2OM_mYUeWBc</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>If You Steal From The American People, You Will Go To Prison</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2OM_mYUeWBc</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>M3XvW1sSs-E</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>No Tax on Overtime: Promises Made, Promises Kept</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M3XvW1sSs-E</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>_MWwc6p33yM</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press at Joint Base Andrews, Oct. 10, 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_MWwc6p33yM</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="n">
+        <v>493</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>kPscOnPqVM4</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 10, 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kPscOnPqVM4</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="n">
+        <v>337</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>X3kk9Oj5o2E</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 9, 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X3kk9Oj5o2E</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="n">
+        <v>367</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>7YPNA4ZHa1o</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Trump Accounts Turn Dreams Into Possibilities</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7YPNA4ZHa1o</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>1rVWXnUlVLM</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 7, 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1rVWXnUlVLM</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>oW-PQlgw1wo</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Delivers Remarks, Oct. 6, 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oW-PQlgw1wo</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="n">
+        <v>3532</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>JThkq_BtykY</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Arrival at the White House, Oct. 6, 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JThkq_BtykY</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="n">
+        <v>206</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>IkYYt1yHxcQ</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 6, 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IkYYt1yHxcQ</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="n">
+        <v>324</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>kuYkk0TxYuM</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 5, 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kuYkk0TxYuM</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="n">
+        <v>833</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ixWToijvWxE</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Americans across the country are thanking President Trump for delivering on No Tax on Tips</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ixWToijvWxE</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>tlYbzF9hSBE</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Gaggles with Press Upon Departure from the White House, Oct. 3, 2026</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tlYbzF9hSBE</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="n">
+        <v>299</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>AVw2HnrbY44</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Minimum Sentences on Fraudsters</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AVw2HnrbY44</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>unassigned_event_lead</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:47:01+00:00</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>low: metadata-only</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:U21"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Module 2 source review queue
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -10,16 +10,18 @@
     <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sources" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Source Directory" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Read me" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="User Instructions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="New White House leads" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Candidate Review" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Read me" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="User Instructions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="New White House leads" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2234,19 +2236,15 @@
           <t>daily</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-15T02:48:14+00:00</t>
-        </is>
-      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>success_metadata_only</t>
+          <t>not_run</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>metadata_endpoint_reached</t>
+          <t>not_independently_checked</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2259,11 +2257,7 @@
           <t>Automated collector currently fetches recent channel upload metadata only. It does not assign event identity or verify video frames.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/gdelt0003/gdelt0003/actions/runs/38672873524</t>
-        </is>
-      </c>
+      <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@WhiteHouse</t>
@@ -2557,19 +2551,15 @@
           <t>daily</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-15T02:48:14+00:00</t>
-        </is>
-      </c>
+      <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>fetch_failed</t>
+          <t>not_connected</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>fetch_failed_check_run_log</t>
+          <t>not_independently_checked</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2582,11 +2572,7 @@
           <t>User-provided Explorer URL. The daily collector queries the public GDELT DOC API for article metadata only; it does not fetch article bodies or verify event facts. A live metadata response was observed during implementation; subsequent validation requests received HTTP 429, so scheduled availability and rate limits remain to be confirmed.</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/gdelt0003/gdelt0003/actions/runs/38672873524</t>
-        </is>
-      </c>
+      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
           <t>https://gdelt.github.io/#api=doc&amp;query=trump%20&amp;contentmode=ArtList&amp;maxrecords=250&amp;sort=DateDesc&amp;format=html&amp;timespan=1w</t>
@@ -3039,20 +3025,18 @@
   <autoFilter ref="A1:O14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3064,7 +3048,919 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="68" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="64" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="100" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Event title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Queue rank (not a trust score)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Current source path</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Publisher</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate title</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Same-event evidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Clean-source status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Observed stream resolution (not thumbnail/source-master resolution)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Difference from official runtime (seconds)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Source provenance / lineage (reported)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence and limitations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>evt-20261006-7794a6967fc9f877</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Delivers Remarks, Oct. 6, 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Moneycontrol</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jAq7oEbw9Hs</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>same_event_contiguous_speech_observed; exact_cue_offset_unverified</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>At approximately 01:00:01 it shows the matched 'Secretary of War' remarks at tighter framing; in-picture m mark present. The camera station and source lineage are unproved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>evt-20261006-7794a6967fc9f877</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Delivers Remarks, Oct. 6, 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Use White House YouTube event anchor for identity; embedded graphics reported, not a clean editing source.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oW-PQlgw1wo</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>verified_event_anchor</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>At approximately 08:15 and 35:07, in-picture lower-third, White House emblem and QR code are visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>evt-20261006-7794a6967fc9f877</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Delivers Remarks, Oct. 6, 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>NDTV Profit</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CRiW-xC_-WU</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>not_matched_to_reference_moment</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Sample at approximately 00:30:01 shows ship/stage and crowd, not the matched speaking moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Associated Press</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>LIVE: Trump hosts a Columbus Day celebration at the White House</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eteny1ES3wk</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>same_speech_moment_observed</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>1920x1080 (HD1080 player decode)</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>3753.621</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>10.379</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>independent_publisher; camera station and source lineage unverified</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Direct moving-frame review at 20:01, 27:01, and 45:01 after selecting the HD1080 rendition; decoded frames are 1920x1080. At 27:01, player CC reads “of monuments, fountains, uh statues. They were all graffiti strewn,” immediately following the White House anchor's 27:01 cue “of Interior. We fixed 82 monuments,” confirming the same event and contiguous speech. No White House banner, emblem, or QR was visible in sampled AP source frames; an AP logo is burned into the lower-right corner in all samples, so this is not watermark-free. Audience heads/phones touch the lower edge at 20:01 and 27:01 but do not obscure the speaker. Framing is similar to the White House feed and does not establish a distinct camera station. At 62:34 (3753.621 seconds), this is about 10 seconds shorter than the 62:44 official video and is not a longer continuous version. Page upload time is not treated as event time; publication metadata is not used to fill the event date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Times Now World</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Columbus Day Celebration coverage</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OysrZCjorfE</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>same_speech_moment_observed_same_angle</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>10141</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>6377</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>syndicated_or_shared_feed; not independent camera evidence</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>At about 25:01 the player CC and moving frame match the White House 27:01 speech about fixing 82 monuments. Framing/background are nearly identical to the White House source, consistent with same-angle feed/syndication, not a proven alternate camera. In-picture White House banner/logo/QR and Times Now brand/subscribe mark are visible; player CC is separate. Not clean and not a verified longer continuous original. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>RSBN</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>FULL EVENT: President Trump Holds Exciting Columbus Day Celebration - 10/09/26</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-6mZSshfpAc</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>same_event_scene_verified; exact_reference_moment_unverified</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>3714</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>same_publisher_lineage_unverified</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>At 22:31 player CC reads a phrase matching the same event speech; White House East Room decor and speaker establish same-event content. Forward medium-close framing resembles the White House view; sample does not establish exact reference cue, independent camera, or continuity. RSBN logo, LIVE/White House label and ticker are in-picture. Browser-decoded rendition 1280x720; not maximum/source-master resolution. 61:54, shorter than the 62:44 official video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>RSBN</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>LIVE REPLAY: President Trump Hosts Columbus Day Celebration at White House - 10/09/26</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Os4aPmvxZjA</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>same_event_context_only; sampled_time_not_matched</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>5516</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>1752</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>same_publisher_lineage_unverified</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>At 20:01 sample shows RSBN pre-event/weather split screen; 30:01 shows live wide shot of the same flags/speaker/event. RSBN logo, LIVE bar and ticker are in-picture; player CC separately showed anthem captions. Sampled moments do not match the White House speech cue; no continuity claim. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Use White House YouTube event anchor for identity; embedded graphics reported, not a clean editing source.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>The White House</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=noI4BbQ2wZQ</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>official_title_and_event_anchor; event_date_time_unverified</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>3764</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>official_source</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Direct moving-frame audit at approximately 20:01, 25:01 and 27:01; the live scene identifies the White House event. In-picture White House emblem, TEXT “POTUS” TO 45470 FOR WHITE HOUSE UPDATES banner and QR were directly visible. At 27:01 YouTube player CC was separately visible. Browser-decoded rendition was 1280x720; not claimed as maximum/source-master resolution. Page publication time is not used as event date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>NBC News</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>LIVE: Trump hosts Columbus Day celebration at White House | NBC News</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OLbQ9L1aoks</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>3750</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>FOX 9 Minneapolis-St. Paul</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>LIVE | President Trump hosts Columbus Day celebration at White House</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=879Q3BNa_KQ</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>4206</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>442</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>same_network_lineage_unverified</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Direct page/oEmbed metadata identifies publisher/title; same listed runtime as FOX6 may indicate a shared feed, but lineage is unverified. No moving frames or matched time reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>FOX6 News Milwaukee</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>LIVE | President Trump hosts Columbus Day celebration at White House</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5kT9wyjoNWA</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>4206</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>442</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Fox News</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>President Trump hosts Columbus Day Celebration at the White House</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Ubivu0AQHXo</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>5032</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>1268</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Moving frames at 20:01, 25:01 and 27:01 show the same East Room event, speaker, audience phones and flags; the 25:01 frame is wider than the White House anchor. YouTube CC is a separate player layer. No persistent in-picture station logo/lower-third was seen in the sampled frames, but the whole video was not checked and cleanliness is unverified. No exact matching spoken cue or independent camera/source lineage established. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>President Trump Hosts a Columbus Day Celebration</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>No suitable alternate verified; this row remains a review lead.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Fox Business</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>President Trump hosts Columbus Day Celebration at the White House</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=27CXvjs7jFY</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>5043</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>1279</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N14"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3119,12 +4015,19 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Candidate Review contains up to ten existing video-source rows per event. Queue order is same-event evidence, clean status, observed stream resolution, duration closeness to the official runtime, then publisher/URL for stable ties. It is not a trust score; unknown resolution is not inferred from thumbnails, and rows are never invented to fill the limit. An alternate is selected only when the same speech moment, clean status, and observed stream resolution are all explicitly recorded. Otherwise the White House YouTube anchor remains the identity reference and is not called clean.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3227,7 +4130,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat: record unassigned user video lead
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AI$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
   </definedNames>
@@ -3048,23 +3048,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:AI15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="68" customWidth="1" min="4" max="4"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="64" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
-    <col width="100" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="58" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="58" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="24" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="38" customWidth="1" min="28" max="28"/>
+    <col width="34" customWidth="1" min="29" max="29"/>
+    <col width="70" customWidth="1" min="30" max="30"/>
+    <col width="28" customWidth="1" min="31" max="31"/>
+    <col width="34" customWidth="1" min="32" max="32"/>
+    <col width="24" customWidth="1" min="33" max="33"/>
+    <col width="30" customWidth="1" min="34" max="34"/>
+    <col width="100" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3135,9 +3156,110 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Embedded graphics / occlusion review</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Reuse rights review</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>User-provided characterization (claim; unverified)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>User subjective rating (not independent score)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>User angle opinion (not verified)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Camera/event-time match</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Camera location</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Camera coordinates WGS84</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Camera azimuth (degrees)</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Camera height (meters)</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Camera pitch (degrees)</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Camera equipment</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Media/camera department</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Publicly confirmed professional crew</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Media-seat annotation</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Camera evidence URL</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Camera method</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Camera uncertainty/error</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Camera confidence</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Camera verification status</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
           <t>Evidence and limitations</t>
         </is>
       </c>
+      <c r="AI1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3193,6 +3315,35 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
           <t>At approximately 01:00:01 it shows the matched 'Secretary of War' remarks at tighter framing; in-picture m mark present. The camera station and source lineage are unproved.</t>
         </is>
       </c>
@@ -3251,6 +3402,35 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr"/>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr">
+        <is>
           <t>At approximately 08:15 and 35:07, in-picture lower-third, White House emblem and QR code are visible.</t>
         </is>
       </c>
@@ -3309,6 +3489,35 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr">
+        <is>
           <t>Sample at approximately 00:30:01 shows ship/stage and crowd, not the matched speaking moment.</t>
         </is>
       </c>
@@ -3371,6 +3580,35 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
+          <t>sampled_at_20:01,27:01,45:01</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="inlineStr"/>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr">
+        <is>
           <t>Direct moving-frame review at 20:01, 27:01, and 45:01 after selecting the HD1080 rendition; decoded frames are 1920x1080. At 27:01, player CC reads “of monuments, fountains, uh statues. They were all graffiti strewn,” immediately following the White House anchor's 27:01 cue “of Interior. We fixed 82 monuments,” confirming the same event and contiguous speech. No White House banner, emblem, or QR was visible in sampled AP source frames; an AP logo is burned into the lower-right corner in all samples, so this is not watermark-free. Audience heads/phones touch the lower edge at 20:01 and 27:01 but do not obscure the speaker. Framing is similar to the White House feed and does not establish a distinct camera station. At 62:34 (3753.621 seconds), this is about 10 seconds shorter than the 62:44 official video and is not a longer continuous version. Page upload time is not treated as event time; publication metadata is not used to fill the event date.</t>
         </is>
       </c>
@@ -3433,6 +3671,35 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
+          <t>sampled_around_25:01</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr"/>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr">
+        <is>
           <t>At about 25:01 the player CC and moving frame match the White House 27:01 speech about fixing 82 monuments. Framing/background are nearly identical to the White House source, consistent with same-angle feed/syndication, not a proven alternate camera. In-picture White House banner/logo/QR and Times Now brand/subscribe mark are visible; player CC is separate. Not clean and not a verified longer continuous original. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
       </c>
@@ -3495,6 +3762,35 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
+          <t>sampled_at_22:31</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr">
+        <is>
           <t>At 22:31 player CC reads a phrase matching the same event speech; White House East Room decor and speaker establish same-event content. Forward medium-close framing resembles the White House view; sample does not establish exact reference cue, independent camera, or continuity. RSBN logo, LIVE/White House label and ticker are in-picture. Browser-decoded rendition 1280x720; not maximum/source-master resolution. 61:54, shorter than the 62:44 official video.</t>
         </is>
       </c>
@@ -3557,6 +3853,35 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
+          <t>sampled_at_20:01,30:01</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr"/>
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AG8" s="2" t="inlineStr"/>
+      <c r="AH8" s="2" t="inlineStr"/>
+      <c r="AI8" s="2" t="inlineStr">
+        <is>
           <t>At 20:01 sample shows RSBN pre-event/weather split screen; 30:01 shows live wide shot of the same flags/speaker/event. RSBN logo, LIVE bar and ticker are in-picture; player CC separately showed anthem captions. Sampled moments do not match the White House speech cue; no continuity claim. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
       </c>
@@ -3619,6 +3944,35 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
+          <t>sampled_at_20:01,25:01,27:01</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr"/>
+      <c r="X9" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AA9" s="2" t="inlineStr"/>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="inlineStr"/>
+      <c r="AG9" s="2" t="inlineStr"/>
+      <c r="AH9" s="2" t="inlineStr"/>
+      <c r="AI9" s="2" t="inlineStr">
+        <is>
           <t>Direct moving-frame audit at approximately 20:01, 25:01 and 27:01; the live scene identifies the White House event. In-picture White House emblem, TEXT “POTUS” TO 45470 FOR WHITE HOUSE UPDATES banner and QR were directly visible. At 27:01 YouTube player CC was separately visible. Browser-decoded rendition was 1280x720; not claimed as maximum/source-master resolution. Page publication time is not used as event date.</t>
         </is>
       </c>
@@ -3681,6 +4035,35 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="inlineStr"/>
+      <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr"/>
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AA10" s="2" t="inlineStr"/>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="inlineStr"/>
+      <c r="AH10" s="2" t="inlineStr"/>
+      <c r="AI10" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
       </c>
@@ -3743,6 +4126,35 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr"/>
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr"/>
+      <c r="Y11" s="2" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AG11" s="2" t="inlineStr"/>
+      <c r="AH11" s="2" t="inlineStr"/>
+      <c r="AI11" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; same listed runtime as FOX6 may indicate a shared feed, but lineage is unverified. No moving frames or matched time reviewed.</t>
         </is>
       </c>
@@ -3805,6 +4217,35 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr"/>
+      <c r="Y12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr"/>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="inlineStr"/>
+      <c r="AH12" s="2" t="inlineStr"/>
+      <c r="AI12" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
       </c>
@@ -3867,6 +4308,35 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
+          <t>sampled_at_20:01,25:01,27:01</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr"/>
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr"/>
+      <c r="Y13" s="2" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr"/>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr"/>
+      <c r="AF13" s="2" t="inlineStr"/>
+      <c r="AG13" s="2" t="inlineStr"/>
+      <c r="AH13" s="2" t="inlineStr"/>
+      <c r="AI13" s="2" t="inlineStr">
+        <is>
           <t>Moving frames at 20:01, 25:01 and 27:01 show the same East Room event, speaker, audience phones and flags; the 25:01 frame is wider than the White House anchor. YouTube CC is a separate player layer. No persistent in-picture station logo/lower-third was seen in the sampled frames, but the whole video was not checked and cleanliness is unverified. No exact matching spoken cue or independent camera/source lineage established. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
       </c>
@@ -3929,12 +4399,196 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
+          <t>metadata_only</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="inlineStr"/>
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr"/>
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr"/>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr"/>
+      <c r="AH14" s="2" t="inlineStr"/>
+      <c r="AI14" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned video lead (event match pending)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned lead only; do not compare or substitute until the exact event and time are independently matched. Do not mix with the October 13 Katie event absent that match.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>not reviewed</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>User-provided YouTube source lead (title not reviewed)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rQlpuY2tj-4</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>pending_manual_review</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_provenance_review</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>这个源可以 更长 干净 高清 可信源,全体通报学习</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>打90分...此角度视频典范,还可以增补其它角度</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>pending_verified_position</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>not_assessed</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AF15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG15" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AH15" s="2" t="inlineStr">
+        <is>
+          <t>URL and characterization supplied by the user. Event match, runtime, actual video-stream resolution, embedded graphics/occlusion, provenance/independence, and reuse rights have not been checked. The characterization is not verified evidence.</t>
+        </is>
+      </c>
+      <c r="AI15" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N14"/>
+  <autoFilter ref="A1:AI15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -3949,6 +4603,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3960,7 +4615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4019,6 +4674,13 @@
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Candidate Review contains up to ten existing video-source rows per event. Queue order is same-event evidence, clean status, observed stream resolution, duration closeness to the official runtime, then publisher/URL for stable ties. It is not a trust score; unknown resolution is not inferred from thumbnails, and rows are never invented to fill the limit. An alternate is selected only when the same speech moment, clean status, and observed stream resolution are all explicitly recorded. Otherwise the White House YouTube anchor remains the identity reference and is not called clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>User-submitted video leads without an exact event/time match appear as unassigned rows. User claims and subjective ratings are not verification. Camera location, coordinates, azimuth, height, pitch, equipment, department, publicly confirmed crew, and media-seat annotations require direct evidence, method, uncertainty, confidence, and a verification status; unknowns remain unknown. Do not infer private identities or mix an unassigned lead into a named event.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: record second unverified video lead
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AI$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AM$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
   </definedNames>
@@ -3048,7 +3048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI15"/>
+  <dimension ref="A1:AM16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3085,7 +3085,11 @@
     <col width="34" customWidth="1" min="32" max="32"/>
     <col width="24" customWidth="1" min="33" max="33"/>
     <col width="30" customWidth="1" min="34" max="34"/>
-    <col width="100" customWidth="1" min="35" max="35"/>
+    <col width="38" customWidth="1" min="35" max="35"/>
+    <col width="30" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="37" max="37"/>
+    <col width="44" customWidth="1" min="38" max="38"/>
+    <col width="100" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3256,10 +3260,30 @@
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
+          <t>Repeated/static-scene review</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Source credibility review</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Independent camera review</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Cross-lead angle/lineage comparison</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
           <t>Evidence and limitations</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="n"/>
+      <c r="AM1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3344,6 +3368,26 @@
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
           <t>At approximately 01:00:01 it shows the matched 'Secretary of War' remarks at tighter framing; in-picture m mark present. The camera station and source lineage are unproved.</t>
         </is>
       </c>
@@ -3431,6 +3475,26 @@
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK3" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
           <t>At approximately 08:15 and 35:07, in-picture lower-third, White House emblem and QR code are visible.</t>
         </is>
       </c>
@@ -3518,6 +3582,26 @@
       <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK4" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL4" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM4" s="2" t="inlineStr">
+        <is>
           <t>Sample at approximately 00:30:01 shows ship/stage and crowd, not the matched speaking moment.</t>
         </is>
       </c>
@@ -3609,6 +3693,26 @@
       <c r="AH5" s="2" t="inlineStr"/>
       <c r="AI5" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK5" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL5" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM5" s="2" t="inlineStr">
+        <is>
           <t>Direct moving-frame review at 20:01, 27:01, and 45:01 after selecting the HD1080 rendition; decoded frames are 1920x1080. At 27:01, player CC reads “of monuments, fountains, uh statues. They were all graffiti strewn,” immediately following the White House anchor's 27:01 cue “of Interior. We fixed 82 monuments,” confirming the same event and contiguous speech. No White House banner, emblem, or QR was visible in sampled AP source frames; an AP logo is burned into the lower-right corner in all samples, so this is not watermark-free. Audience heads/phones touch the lower edge at 20:01 and 27:01 but do not obscure the speaker. Framing is similar to the White House feed and does not establish a distinct camera station. At 62:34 (3753.621 seconds), this is about 10 seconds shorter than the 62:44 official video and is not a longer continuous version. Page upload time is not treated as event time; publication metadata is not used to fill the event date.</t>
         </is>
       </c>
@@ -3700,6 +3804,26 @@
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK6" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM6" s="2" t="inlineStr">
+        <is>
           <t>At about 25:01 the player CC and moving frame match the White House 27:01 speech about fixing 82 monuments. Framing/background are nearly identical to the White House source, consistent with same-angle feed/syndication, not a proven alternate camera. In-picture White House banner/logo/QR and Times Now brand/subscribe mark are visible; player CC is separate. Not clean and not a verified longer continuous original. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
       </c>
@@ -3791,6 +3915,26 @@
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK7" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL7" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM7" s="2" t="inlineStr">
+        <is>
           <t>At 22:31 player CC reads a phrase matching the same event speech; White House East Room decor and speaker establish same-event content. Forward medium-close framing resembles the White House view; sample does not establish exact reference cue, independent camera, or continuity. RSBN logo, LIVE/White House label and ticker are in-picture. Browser-decoded rendition 1280x720; not maximum/source-master resolution. 61:54, shorter than the 62:44 official video.</t>
         </is>
       </c>
@@ -3882,6 +4026,26 @@
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK8" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL8" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM8" s="2" t="inlineStr">
+        <is>
           <t>At 20:01 sample shows RSBN pre-event/weather split screen; 30:01 shows live wide shot of the same flags/speaker/event. RSBN logo, LIVE bar and ticker are in-picture; player CC separately showed anthem captions. Sampled moments do not match the White House speech cue; no continuity claim. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
       </c>
@@ -3973,6 +4137,26 @@
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK9" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL9" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM9" s="2" t="inlineStr">
+        <is>
           <t>Direct moving-frame audit at approximately 20:01, 25:01 and 27:01; the live scene identifies the White House event. In-picture White House emblem, TEXT “POTUS” TO 45470 FOR WHITE HOUSE UPDATES banner and QR were directly visible. At 27:01 YouTube player CC was separately visible. Browser-decoded rendition was 1280x720; not claimed as maximum/source-master resolution. Page publication time is not used as event date.</t>
         </is>
       </c>
@@ -4064,6 +4248,26 @@
       <c r="AH10" s="2" t="inlineStr"/>
       <c r="AI10" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ10" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK10" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL10" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM10" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
       </c>
@@ -4155,6 +4359,26 @@
       <c r="AH11" s="2" t="inlineStr"/>
       <c r="AI11" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ11" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK11" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL11" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM11" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; same listed runtime as FOX6 may indicate a shared feed, but lineage is unverified. No moving frames or matched time reviewed.</t>
         </is>
       </c>
@@ -4246,6 +4470,26 @@
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ12" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK12" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL12" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM12" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
       </c>
@@ -4337,6 +4581,26 @@
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ13" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK13" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL13" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM13" s="2" t="inlineStr">
+        <is>
           <t>Moving frames at 20:01, 25:01 and 27:01 show the same East Room event, speaker, audience phones and flags; the 25:01 frame is wider than the White House anchor. YouTube CC is a separate player layer. No persistent in-picture station logo/lower-third was seen in the sampled frames, but the whole video was not checked and cleanliness is unverified. No exact matching spoken cue or independent camera/source lineage established. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
       </c>
@@ -4428,6 +4692,26 @@
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ14" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK14" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL14" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AM14" s="2" t="inlineStr">
+        <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
       </c>
@@ -4582,13 +4866,204 @@
       </c>
       <c r="AH15" s="2" t="inlineStr">
         <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AI15" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AK15" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AL15" s="2" t="inlineStr">
+        <is>
           <t>URL and characterization supplied by the user. Event match, runtime, actual video-stream resolution, embedded graphics/occlusion, provenance/independence, and reuse rights have not been checked. The characterization is not verified evidence.</t>
         </is>
       </c>
-      <c r="AI15" s="2" t="n"/>
+      <c r="AM15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned video lead (event match pending)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned lead only; do not compare or substitute until the exact event and time are independently matched. Do not mix with the October 13 Katie event absent that match.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>not reviewed</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>User-provided YouTube source lead (title not reviewed)</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=UgIivPOerNc</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_provenance_review</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>此链接50 分 虽然长 但是台标信号凑数 不变风景凑 还有logo 还有横幅遮挡</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>pending_verified_position</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr">
+        <is>
+          <t>not_assessed</t>
+        </is>
+      </c>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AF16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG16" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AH16" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AI16" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AJ16" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AK16" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
+      <c r="AL16" s="2" t="inlineStr">
+        <is>
+          <t>User reports a long runtime may include station/signal idents or repeated static scenes, with a logo and banner obscuring the picture. These observations are not independently verified. Assess runtime and repetition separately; do not rank by duration alone. Confirm exact event and time before comparing with rQlpuY2tj-4; do not assume the same event or a different camera angle. Actual stream resolution, source credibility, independent camera status, lineage, graphics, and reuse rights remain unverified.</t>
+        </is>
+      </c>
+      <c r="AM16" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI15"/>
+  <autoFilter ref="A1:AM16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -4604,6 +5079,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4615,7 +5091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4681,6 +5157,13 @@
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>User-submitted video leads without an exact event/time match appear as unassigned rows. User claims and subjective ratings are not verification. Camera location, coordinates, azimuth, height, pitch, equipment, department, publicly confirmed crew, and media-seat annotations require direct evidence, method, uncertainty, confidence, and a verification status; unknowns remain unknown. Do not infer private identities or mix an unassigned lead into a named event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Do not rank a source as superior based on runtime alone. Assess repeated/static scenes, embedded logos/banners, actual stream resolution, exact event/time match, source credibility, independent camera status, and source lineage separately. Comparing two user-submitted links requires first confirming the same event/time and then checking angle and lineage; neither same-event nor different-angle status is assumed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: record third unverified video lead
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AM$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AN$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
   </definedNames>
@@ -3048,7 +3048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM16"/>
+  <dimension ref="A1:AN17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3068,28 +3068,29 @@
     <col width="28" customWidth="1" min="15" max="15"/>
     <col width="58" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="58" customWidth="1" min="18" max="18"/>
-    <col width="40" customWidth="1" min="19" max="19"/>
-    <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="28" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="58" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="42" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="22" max="22"/>
     <col width="24" customWidth="1" min="23" max="23"/>
     <col width="24" customWidth="1" min="24" max="24"/>
     <col width="24" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
     <col width="30" customWidth="1" min="27" max="27"/>
-    <col width="38" customWidth="1" min="28" max="28"/>
-    <col width="34" customWidth="1" min="29" max="29"/>
-    <col width="70" customWidth="1" min="30" max="30"/>
-    <col width="28" customWidth="1" min="31" max="31"/>
-    <col width="34" customWidth="1" min="32" max="32"/>
-    <col width="24" customWidth="1" min="33" max="33"/>
-    <col width="30" customWidth="1" min="34" max="34"/>
-    <col width="38" customWidth="1" min="35" max="35"/>
-    <col width="30" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
+    <col width="38" customWidth="1" min="29" max="29"/>
+    <col width="34" customWidth="1" min="30" max="30"/>
+    <col width="70" customWidth="1" min="31" max="31"/>
+    <col width="28" customWidth="1" min="32" max="32"/>
+    <col width="34" customWidth="1" min="33" max="33"/>
+    <col width="24" customWidth="1" min="34" max="34"/>
+    <col width="30" customWidth="1" min="35" max="35"/>
+    <col width="38" customWidth="1" min="36" max="36"/>
     <col width="30" customWidth="1" min="37" max="37"/>
-    <col width="44" customWidth="1" min="38" max="38"/>
-    <col width="100" customWidth="1" min="39" max="39"/>
+    <col width="30" customWidth="1" min="38" max="38"/>
+    <col width="44" customWidth="1" min="39" max="39"/>
+    <col width="100" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3180,110 +3181,115 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>User feature score (not independent; rubric unspecified)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>User angle opinion (not verified)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Camera/event-time match</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Camera location</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Camera coordinates WGS84</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Camera azimuth (degrees)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Camera height (meters)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Camera pitch (degrees)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Camera equipment</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Media/camera department</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Publicly confirmed professional crew</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Media-seat annotation</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Camera evidence URL</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Camera method</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Camera uncertainty/error</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Camera confidence</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Camera verification status</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Repeated/static-scene review</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Source credibility review</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Independent camera review</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Cross-lead angle/lineage comparison</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Evidence and limitations</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="n"/>
+      <c r="AN1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3366,27 +3372,28 @@
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
       <c r="AH2" s="2" t="inlineStr"/>
-      <c r="AI2" s="2" t="inlineStr">
+      <c r="AI2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr">
+      <c r="AK2" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AL2" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL2" s="2" t="inlineStr">
+      <c r="AM2" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>At approximately 01:00:01 it shows the matched 'Secretary of War' remarks at tighter framing; in-picture m mark present. The camera station and source lineage are unproved.</t>
         </is>
@@ -3473,27 +3480,28 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
-      <c r="AI3" s="2" t="inlineStr">
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr">
+      <c r="AK3" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK3" s="2" t="inlineStr">
+      <c r="AL3" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL3" s="2" t="inlineStr">
+      <c r="AM3" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM3" s="2" t="inlineStr">
+      <c r="AN3" s="2" t="inlineStr">
         <is>
           <t>At approximately 08:15 and 35:07, in-picture lower-third, White House emblem and QR code are visible.</t>
         </is>
@@ -3580,27 +3588,28 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
-      <c r="AI4" s="2" t="inlineStr">
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr">
+      <c r="AK4" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK4" s="2" t="inlineStr">
+      <c r="AL4" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL4" s="2" t="inlineStr">
+      <c r="AM4" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM4" s="2" t="inlineStr">
+      <c r="AN4" s="2" t="inlineStr">
         <is>
           <t>Sample at approximately 00:30:01 shows ship/stage and crowd, not the matched speaking moment.</t>
         </is>
@@ -3691,27 +3700,28 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
-      <c r="AI5" s="2" t="inlineStr">
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr">
+      <c r="AK5" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK5" s="2" t="inlineStr">
+      <c r="AL5" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL5" s="2" t="inlineStr">
+      <c r="AM5" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM5" s="2" t="inlineStr">
+      <c r="AN5" s="2" t="inlineStr">
         <is>
           <t>Direct moving-frame review at 20:01, 27:01, and 45:01 after selecting the HD1080 rendition; decoded frames are 1920x1080. At 27:01, player CC reads “of monuments, fountains, uh statues. They were all graffiti strewn,” immediately following the White House anchor's 27:01 cue “of Interior. We fixed 82 monuments,” confirming the same event and contiguous speech. No White House banner, emblem, or QR was visible in sampled AP source frames; an AP logo is burned into the lower-right corner in all samples, so this is not watermark-free. Audience heads/phones touch the lower edge at 20:01 and 27:01 but do not obscure the speaker. Framing is similar to the White House feed and does not establish a distinct camera station. At 62:34 (3753.621 seconds), this is about 10 seconds shorter than the 62:44 official video and is not a longer continuous version. Page upload time is not treated as event time; publication metadata is not used to fill the event date.</t>
         </is>
@@ -3802,27 +3812,28 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
-      <c r="AI6" s="2" t="inlineStr">
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr">
+      <c r="AK6" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK6" s="2" t="inlineStr">
+      <c r="AL6" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL6" s="2" t="inlineStr">
+      <c r="AM6" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM6" s="2" t="inlineStr">
+      <c r="AN6" s="2" t="inlineStr">
         <is>
           <t>At about 25:01 the player CC and moving frame match the White House 27:01 speech about fixing 82 monuments. Framing/background are nearly identical to the White House source, consistent with same-angle feed/syndication, not a proven alternate camera. In-picture White House banner/logo/QR and Times Now brand/subscribe mark are visible; player CC is separate. Not clean and not a verified longer continuous original. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
@@ -3913,27 +3924,28 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
-      <c r="AI7" s="2" t="inlineStr">
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr">
+      <c r="AK7" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK7" s="2" t="inlineStr">
+      <c r="AL7" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL7" s="2" t="inlineStr">
+      <c r="AM7" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM7" s="2" t="inlineStr">
+      <c r="AN7" s="2" t="inlineStr">
         <is>
           <t>At 22:31 player CC reads a phrase matching the same event speech; White House East Room decor and speaker establish same-event content. Forward medium-close framing resembles the White House view; sample does not establish exact reference cue, independent camera, or continuity. RSBN logo, LIVE/White House label and ticker are in-picture. Browser-decoded rendition 1280x720; not maximum/source-master resolution. 61:54, shorter than the 62:44 official video.</t>
         </is>
@@ -4024,27 +4036,28 @@
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
-      <c r="AI8" s="2" t="inlineStr">
+      <c r="AI8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr">
+      <c r="AK8" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK8" s="2" t="inlineStr">
+      <c r="AL8" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL8" s="2" t="inlineStr">
+      <c r="AM8" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM8" s="2" t="inlineStr">
+      <c r="AN8" s="2" t="inlineStr">
         <is>
           <t>At 20:01 sample shows RSBN pre-event/weather split screen; 30:01 shows live wide shot of the same flags/speaker/event. RSBN logo, LIVE bar and ticker are in-picture; player CC separately showed anthem captions. Sampled moments do not match the White House speech cue; no continuity claim. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
@@ -4135,27 +4148,28 @@
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
-      <c r="AI9" s="2" t="inlineStr">
+      <c r="AI9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ9" s="2" t="inlineStr">
+      <c r="AK9" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK9" s="2" t="inlineStr">
+      <c r="AL9" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL9" s="2" t="inlineStr">
+      <c r="AM9" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM9" s="2" t="inlineStr">
+      <c r="AN9" s="2" t="inlineStr">
         <is>
           <t>Direct moving-frame audit at approximately 20:01, 25:01 and 27:01; the live scene identifies the White House event. In-picture White House emblem, TEXT “POTUS” TO 45470 FOR WHITE HOUSE UPDATES banner and QR were directly visible. At 27:01 YouTube player CC was separately visible. Browser-decoded rendition was 1280x720; not claimed as maximum/source-master resolution. Page publication time is not used as event date.</t>
         </is>
@@ -4246,27 +4260,28 @@
       <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr"/>
-      <c r="AI10" s="2" t="inlineStr">
+      <c r="AI10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ10" s="2" t="inlineStr">
+      <c r="AK10" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK10" s="2" t="inlineStr">
+      <c r="AL10" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL10" s="2" t="inlineStr">
+      <c r="AM10" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM10" s="2" t="inlineStr">
+      <c r="AN10" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
@@ -4357,27 +4372,28 @@
       <c r="AF11" s="2" t="inlineStr"/>
       <c r="AG11" s="2" t="inlineStr"/>
       <c r="AH11" s="2" t="inlineStr"/>
-      <c r="AI11" s="2" t="inlineStr">
+      <c r="AI11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ11" s="2" t="inlineStr">
+      <c r="AK11" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK11" s="2" t="inlineStr">
+      <c r="AL11" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL11" s="2" t="inlineStr">
+      <c r="AM11" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM11" s="2" t="inlineStr">
+      <c r="AN11" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; same listed runtime as FOX6 may indicate a shared feed, but lineage is unverified. No moving frames or matched time reviewed.</t>
         </is>
@@ -4468,27 +4484,28 @@
       <c r="AF12" s="2" t="inlineStr"/>
       <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr"/>
-      <c r="AI12" s="2" t="inlineStr">
+      <c r="AI12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ12" s="2" t="inlineStr">
+      <c r="AK12" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK12" s="2" t="inlineStr">
+      <c r="AL12" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL12" s="2" t="inlineStr">
+      <c r="AM12" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM12" s="2" t="inlineStr">
+      <c r="AN12" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
@@ -4579,27 +4596,28 @@
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="inlineStr"/>
       <c r="AH13" s="2" t="inlineStr"/>
-      <c r="AI13" s="2" t="inlineStr">
+      <c r="AI13" s="2" t="inlineStr"/>
+      <c r="AJ13" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ13" s="2" t="inlineStr">
+      <c r="AK13" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK13" s="2" t="inlineStr">
+      <c r="AL13" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL13" s="2" t="inlineStr">
+      <c r="AM13" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM13" s="2" t="inlineStr">
+      <c r="AN13" s="2" t="inlineStr">
         <is>
           <t>Moving frames at 20:01, 25:01 and 27:01 show the same East Room event, speaker, audience phones and flags; the 25:01 frame is wider than the White House anchor. YouTube CC is a separate player layer. No persistent in-picture station logo/lower-third was seen in the sampled frames, but the whole video was not checked and cleanliness is unverified. No exact matching spoken cue or independent camera/source lineage established. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
@@ -4690,27 +4708,28 @@
       <c r="AF14" s="2" t="inlineStr"/>
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
-      <c r="AI14" s="2" t="inlineStr">
+      <c r="AI14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ14" s="2" t="inlineStr">
+      <c r="AK14" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK14" s="2" t="inlineStr">
+      <c r="AL14" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL14" s="2" t="inlineStr">
+      <c r="AM14" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM14" s="2" t="inlineStr">
+      <c r="AN14" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
@@ -4788,108 +4807,109 @@
       <c r="Q15" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="R15" s="2" t="inlineStr">
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
         <is>
           <t>打90分...此角度视频典范,还可以增补其它角度</t>
         </is>
       </c>
-      <c r="S15" s="2" t="inlineStr">
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_and_time_match</t>
         </is>
       </c>
-      <c r="T15" s="2" t="inlineStr">
+      <c r="U15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="U15" s="2" t="inlineStr">
+      <c r="V15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="V15" s="2" t="inlineStr">
+      <c r="W15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="W15" s="2" t="inlineStr">
+      <c r="X15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="X15" s="2" t="inlineStr">
+      <c r="Y15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="inlineStr">
+      <c r="Z15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="Z15" s="2" t="inlineStr">
+      <c r="AA15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="inlineStr">
+      <c r="AB15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB15" s="2" t="inlineStr">
+      <c r="AC15" s="2" t="inlineStr">
         <is>
           <t>pending_verified_position</t>
         </is>
       </c>
-      <c r="AC15" s="2" t="inlineStr"/>
-      <c r="AD15" s="2" t="inlineStr">
+      <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr">
         <is>
           <t>not_assessed</t>
         </is>
       </c>
-      <c r="AE15" s="2" t="inlineStr">
+      <c r="AF15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AF15" s="2" t="inlineStr">
+      <c r="AG15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AG15" s="2" t="inlineStr">
+      <c r="AH15" s="2" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="AH15" s="2" t="inlineStr">
+      <c r="AI15" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AI15" s="2" t="inlineStr">
+      <c r="AJ15" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AJ15" s="2" t="inlineStr">
+      <c r="AK15" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AK15" s="2" t="inlineStr">
+      <c r="AL15" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AL15" s="2" t="inlineStr">
+      <c r="AM15" s="2" t="inlineStr">
         <is>
           <t>URL and characterization supplied by the user. Event match, runtime, actual video-stream resolution, embedded graphics/occlusion, provenance/independence, and reuse rights have not been checked. The characterization is not verified evidence.</t>
         </is>
       </c>
-      <c r="AM15" s="2" t="n"/>
+      <c r="AN15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr"/>
@@ -4964,106 +4984,285 @@
         <v>50</v>
       </c>
       <c r="R16" s="2" t="inlineStr"/>
-      <c r="S16" s="2" t="inlineStr">
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_and_time_match</t>
         </is>
       </c>
-      <c r="T16" s="2" t="inlineStr">
+      <c r="U16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="U16" s="2" t="inlineStr">
+      <c r="V16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="V16" s="2" t="inlineStr">
+      <c r="W16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="W16" s="2" t="inlineStr">
+      <c r="X16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="X16" s="2" t="inlineStr">
+      <c r="Y16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="Y16" s="2" t="inlineStr">
+      <c r="Z16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="Z16" s="2" t="inlineStr">
+      <c r="AA16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AA16" s="2" t="inlineStr">
+      <c r="AB16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB16" s="2" t="inlineStr">
+      <c r="AC16" s="2" t="inlineStr">
         <is>
           <t>pending_verified_position</t>
         </is>
       </c>
-      <c r="AC16" s="2" t="inlineStr"/>
-      <c r="AD16" s="2" t="inlineStr">
+      <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr">
         <is>
           <t>not_assessed</t>
         </is>
       </c>
-      <c r="AE16" s="2" t="inlineStr">
+      <c r="AF16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AF16" s="2" t="inlineStr">
+      <c r="AG16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="AG16" s="2" t="inlineStr">
+      <c r="AH16" s="2" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="AH16" s="2" t="inlineStr">
+      <c r="AI16" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AI16" s="2" t="inlineStr">
+      <c r="AJ16" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AJ16" s="2" t="inlineStr">
+      <c r="AK16" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AK16" s="2" t="inlineStr">
+      <c r="AL16" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AL16" s="2" t="inlineStr">
+      <c r="AM16" s="2" t="inlineStr">
         <is>
           <t>User reports a long runtime may include station/signal idents or repeated static scenes, with a logo and banner obscuring the picture. These observations are not independently verified. Assess runtime and repetition separately; do not rank by duration alone. Confirm exact event and time before comparing with rQlpuY2tj-4; do not assume the same event or a different camera angle. Actual stream resolution, source credibility, independent camera status, lineage, graphics, and reuse rights remain unverified.</t>
         </is>
       </c>
-      <c r="AM16" s="2" t="n"/>
+      <c r="AN16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned video lead (event match pending)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned lead only; do not compare or substitute until the exact event and time are independently matched. Do not mix with the October 13 Katie event absent that match.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>not reviewed</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>User-provided YouTube source lead (title not reviewed)</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Uya88MLbHV0</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_provenance_review</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>此时长一版 和白宫官方类似 横幅过大 但是特色是由不同角度 整体50分 其中特色分10分</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>用户认为特色是由不同角度；是否为独立摄像机位尚未核实。</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>pending_verified_position</t>
+        </is>
+      </c>
+      <c r="AD17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
+          <t>not_assessed</t>
+        </is>
+      </c>
+      <c r="AF17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AH17" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AI17" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AJ17" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AK17" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AL17" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_match_people_stage_background_audio_continuity_and_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AM17" s="2" t="inlineStr">
+        <is>
+          <t>User characterizes the source as a long-form version similar to the White House official and reports a large banner and different angles. These are unverified user observations, not established event match, camera independence, or source lineage. Confirm exact event/time, people, stage/background, audio continuity, views, and repost/source lineage before comparing with rQlpuY2tj-4 or UgIivPOerNc. Duration, actual resolution, credibility, graphics, lineage, and reuse rights remain unverified. The user's overall and feature scores are subjective; the remaining rubric components and scale are unspecified.</t>
+        </is>
+      </c>
+      <c r="AN17" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM16"/>
+  <autoFilter ref="A1:AN17"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -5080,6 +5279,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: record background video source lead
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AN$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$AP$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'User Instructions'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'New White House leads'!$A$1:$U$21</definedName>
   </definedNames>
@@ -3048,7 +3048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN17"/>
+  <dimension ref="A1:AP18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3090,7 +3090,9 @@
     <col width="30" customWidth="1" min="37" max="37"/>
     <col width="30" customWidth="1" min="38" max="38"/>
     <col width="44" customWidth="1" min="39" max="39"/>
-    <col width="100" customWidth="1" min="40" max="40"/>
+    <col width="68" customWidth="1" min="40" max="40"/>
+    <col width="92" customWidth="1" min="41" max="41"/>
+    <col width="100" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3186,110 +3188,120 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>User-proposed role (not verified)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>User-requested follow-up (pending)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>User angle opinion (not verified)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Camera/event-time match</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Camera location</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Camera coordinates WGS84</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Camera azimuth (degrees)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Camera height (meters)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Camera pitch (degrees)</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Camera equipment</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Media/camera department</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Publicly confirmed professional crew</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Media-seat annotation</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Camera evidence URL</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Camera method</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Camera uncertainty/error</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Camera confidence</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Camera verification status</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Repeated/static-scene review</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Source credibility review</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Independent camera review</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Cross-lead angle/lineage comparison</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Evidence and limitations</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="n"/>
+      <c r="AP1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3373,27 +3385,29 @@
       <c r="AG2" s="2" t="inlineStr"/>
       <c r="AH2" s="2" t="inlineStr"/>
       <c r="AI2" s="2" t="inlineStr"/>
-      <c r="AJ2" s="2" t="inlineStr">
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="inlineStr"/>
+      <c r="AL2" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AM2" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL2" s="2" t="inlineStr">
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
+      <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN2" s="2" t="inlineStr">
+      <c r="AP2" s="2" t="inlineStr">
         <is>
           <t>At approximately 01:00:01 it shows the matched 'Secretary of War' remarks at tighter framing; in-picture m mark present. The camera station and source lineage are unproved.</t>
         </is>
@@ -3481,27 +3495,29 @@
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
-      <c r="AJ3" s="2" t="inlineStr">
+      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AK3" s="2" t="inlineStr"/>
+      <c r="AL3" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK3" s="2" t="inlineStr">
+      <c r="AM3" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL3" s="2" t="inlineStr">
+      <c r="AN3" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM3" s="2" t="inlineStr">
+      <c r="AO3" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN3" s="2" t="inlineStr">
+      <c r="AP3" s="2" t="inlineStr">
         <is>
           <t>At approximately 08:15 and 35:07, in-picture lower-third, White House emblem and QR code are visible.</t>
         </is>
@@ -3589,27 +3605,29 @@
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
       <c r="AI4" s="2" t="inlineStr"/>
-      <c r="AJ4" s="2" t="inlineStr">
+      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AK4" s="2" t="inlineStr"/>
+      <c r="AL4" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK4" s="2" t="inlineStr">
+      <c r="AM4" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL4" s="2" t="inlineStr">
+      <c r="AN4" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM4" s="2" t="inlineStr">
+      <c r="AO4" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN4" s="2" t="inlineStr">
+      <c r="AP4" s="2" t="inlineStr">
         <is>
           <t>Sample at approximately 00:30:01 shows ship/stage and crowd, not the matched speaking moment.</t>
         </is>
@@ -3701,27 +3719,29 @@
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
       <c r="AI5" s="2" t="inlineStr"/>
-      <c r="AJ5" s="2" t="inlineStr">
+      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AK5" s="2" t="inlineStr"/>
+      <c r="AL5" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK5" s="2" t="inlineStr">
+      <c r="AM5" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL5" s="2" t="inlineStr">
+      <c r="AN5" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM5" s="2" t="inlineStr">
+      <c r="AO5" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN5" s="2" t="inlineStr">
+      <c r="AP5" s="2" t="inlineStr">
         <is>
           <t>Direct moving-frame review at 20:01, 27:01, and 45:01 after selecting the HD1080 rendition; decoded frames are 1920x1080. At 27:01, player CC reads “of monuments, fountains, uh statues. They were all graffiti strewn,” immediately following the White House anchor's 27:01 cue “of Interior. We fixed 82 monuments,” confirming the same event and contiguous speech. No White House banner, emblem, or QR was visible in sampled AP source frames; an AP logo is burned into the lower-right corner in all samples, so this is not watermark-free. Audience heads/phones touch the lower edge at 20:01 and 27:01 but do not obscure the speaker. Framing is similar to the White House feed and does not establish a distinct camera station. At 62:34 (3753.621 seconds), this is about 10 seconds shorter than the 62:44 official video and is not a longer continuous version. Page upload time is not treated as event time; publication metadata is not used to fill the event date.</t>
         </is>
@@ -3813,27 +3833,29 @@
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
       <c r="AI6" s="2" t="inlineStr"/>
-      <c r="AJ6" s="2" t="inlineStr">
+      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AK6" s="2" t="inlineStr"/>
+      <c r="AL6" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK6" s="2" t="inlineStr">
+      <c r="AM6" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL6" s="2" t="inlineStr">
+      <c r="AN6" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM6" s="2" t="inlineStr">
+      <c r="AO6" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN6" s="2" t="inlineStr">
+      <c r="AP6" s="2" t="inlineStr">
         <is>
           <t>At about 25:01 the player CC and moving frame match the White House 27:01 speech about fixing 82 monuments. Framing/background are nearly identical to the White House source, consistent with same-angle feed/syndication, not a proven alternate camera. In-picture White House banner/logo/QR and Times Now brand/subscribe mark are visible; player CC is separate. Not clean and not a verified longer continuous original. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
@@ -3925,27 +3947,29 @@
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
       <c r="AI7" s="2" t="inlineStr"/>
-      <c r="AJ7" s="2" t="inlineStr">
+      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AK7" s="2" t="inlineStr"/>
+      <c r="AL7" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK7" s="2" t="inlineStr">
+      <c r="AM7" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL7" s="2" t="inlineStr">
+      <c r="AN7" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM7" s="2" t="inlineStr">
+      <c r="AO7" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN7" s="2" t="inlineStr">
+      <c r="AP7" s="2" t="inlineStr">
         <is>
           <t>At 22:31 player CC reads a phrase matching the same event speech; White House East Room decor and speaker establish same-event content. Forward medium-close framing resembles the White House view; sample does not establish exact reference cue, independent camera, or continuity. RSBN logo, LIVE/White House label and ticker are in-picture. Browser-decoded rendition 1280x720; not maximum/source-master resolution. 61:54, shorter than the 62:44 official video.</t>
         </is>
@@ -4037,27 +4061,29 @@
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
       <c r="AI8" s="2" t="inlineStr"/>
-      <c r="AJ8" s="2" t="inlineStr">
+      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AK8" s="2" t="inlineStr"/>
+      <c r="AL8" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK8" s="2" t="inlineStr">
+      <c r="AM8" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL8" s="2" t="inlineStr">
+      <c r="AN8" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM8" s="2" t="inlineStr">
+      <c r="AO8" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN8" s="2" t="inlineStr">
+      <c r="AP8" s="2" t="inlineStr">
         <is>
           <t>At 20:01 sample shows RSBN pre-event/weather split screen; 30:01 shows live wide shot of the same flags/speaker/event. RSBN logo, LIVE bar and ticker are in-picture; player CC separately showed anthem captions. Sampled moments do not match the White House speech cue; no continuity claim. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
@@ -4149,27 +4175,29 @@
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
       <c r="AI9" s="2" t="inlineStr"/>
-      <c r="AJ9" s="2" t="inlineStr">
+      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AK9" s="2" t="inlineStr"/>
+      <c r="AL9" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK9" s="2" t="inlineStr">
+      <c r="AM9" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL9" s="2" t="inlineStr">
+      <c r="AN9" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM9" s="2" t="inlineStr">
+      <c r="AO9" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN9" s="2" t="inlineStr">
+      <c r="AP9" s="2" t="inlineStr">
         <is>
           <t>Direct moving-frame audit at approximately 20:01, 25:01 and 27:01; the live scene identifies the White House event. In-picture White House emblem, TEXT “POTUS” TO 45470 FOR WHITE HOUSE UPDATES banner and QR were directly visible. At 27:01 YouTube player CC was separately visible. Browser-decoded rendition was 1280x720; not claimed as maximum/source-master resolution. Page publication time is not used as event date.</t>
         </is>
@@ -4261,27 +4289,29 @@
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr"/>
       <c r="AI10" s="2" t="inlineStr"/>
-      <c r="AJ10" s="2" t="inlineStr">
+      <c r="AJ10" s="2" t="inlineStr"/>
+      <c r="AK10" s="2" t="inlineStr"/>
+      <c r="AL10" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK10" s="2" t="inlineStr">
+      <c r="AM10" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL10" s="2" t="inlineStr">
+      <c r="AN10" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM10" s="2" t="inlineStr">
+      <c r="AO10" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN10" s="2" t="inlineStr">
+      <c r="AP10" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
@@ -4373,27 +4403,29 @@
       <c r="AG11" s="2" t="inlineStr"/>
       <c r="AH11" s="2" t="inlineStr"/>
       <c r="AI11" s="2" t="inlineStr"/>
-      <c r="AJ11" s="2" t="inlineStr">
+      <c r="AJ11" s="2" t="inlineStr"/>
+      <c r="AK11" s="2" t="inlineStr"/>
+      <c r="AL11" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK11" s="2" t="inlineStr">
+      <c r="AM11" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL11" s="2" t="inlineStr">
+      <c r="AN11" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM11" s="2" t="inlineStr">
+      <c r="AO11" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN11" s="2" t="inlineStr">
+      <c r="AP11" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; same listed runtime as FOX6 may indicate a shared feed, but lineage is unverified. No moving frames or matched time reviewed.</t>
         </is>
@@ -4485,27 +4517,29 @@
       <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr"/>
       <c r="AI12" s="2" t="inlineStr"/>
-      <c r="AJ12" s="2" t="inlineStr">
+      <c r="AJ12" s="2" t="inlineStr"/>
+      <c r="AK12" s="2" t="inlineStr"/>
+      <c r="AL12" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK12" s="2" t="inlineStr">
+      <c r="AM12" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL12" s="2" t="inlineStr">
+      <c r="AN12" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM12" s="2" t="inlineStr">
+      <c r="AO12" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN12" s="2" t="inlineStr">
+      <c r="AP12" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
@@ -4597,27 +4631,29 @@
       <c r="AG13" s="2" t="inlineStr"/>
       <c r="AH13" s="2" t="inlineStr"/>
       <c r="AI13" s="2" t="inlineStr"/>
-      <c r="AJ13" s="2" t="inlineStr">
+      <c r="AJ13" s="2" t="inlineStr"/>
+      <c r="AK13" s="2" t="inlineStr"/>
+      <c r="AL13" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK13" s="2" t="inlineStr">
+      <c r="AM13" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL13" s="2" t="inlineStr">
+      <c r="AN13" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM13" s="2" t="inlineStr">
+      <c r="AO13" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN13" s="2" t="inlineStr">
+      <c r="AP13" s="2" t="inlineStr">
         <is>
           <t>Moving frames at 20:01, 25:01 and 27:01 show the same East Room event, speaker, audience phones and flags; the 25:01 frame is wider than the White House anchor. YouTube CC is a separate player layer. No persistent in-picture station logo/lower-third was seen in the sampled frames, but the whole video was not checked and cleanliness is unverified. No exact matching spoken cue or independent camera/source lineage established. Browser-decoded rendition 1280x720; not maximum/source-master resolution.</t>
         </is>
@@ -4709,27 +4745,29 @@
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
       <c r="AI14" s="2" t="inlineStr"/>
-      <c r="AJ14" s="2" t="inlineStr">
+      <c r="AJ14" s="2" t="inlineStr"/>
+      <c r="AK14" s="2" t="inlineStr"/>
+      <c r="AL14" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AK14" s="2" t="inlineStr">
+      <c r="AM14" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AL14" s="2" t="inlineStr">
+      <c r="AN14" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM14" s="2" t="inlineStr">
+      <c r="AO14" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AN14" s="2" t="inlineStr">
+      <c r="AP14" s="2" t="inlineStr">
         <is>
           <t>Direct page/oEmbed metadata identifies publisher/title; no moving frames, matched timestamp, graphics, or footage lineage reviewed.</t>
         </is>
@@ -4808,26 +4846,18 @@
         <v>90</v>
       </c>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr">
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
         <is>
           <t>打90分...此角度视频典范,还可以增补其它角度</t>
         </is>
       </c>
-      <c r="T15" s="2" t="inlineStr">
+      <c r="V15" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_and_time_match</t>
         </is>
       </c>
-      <c r="U15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="V15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -4860,56 +4890,66 @@
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
           <t>pending_verified_position</t>
         </is>
       </c>
-      <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr">
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr">
         <is>
           <t>not_assessed</t>
         </is>
       </c>
-      <c r="AF15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="AH15" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AI15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="AI15" s="2" t="inlineStr">
+      <c r="AK15" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ15" s="2" t="inlineStr">
+      <c r="AL15" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK15" s="2" t="inlineStr">
+      <c r="AM15" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL15" s="2" t="inlineStr">
+      <c r="AN15" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM15" s="2" t="inlineStr">
+      <c r="AO15" s="2" t="inlineStr">
         <is>
           <t>URL and characterization supplied by the user. Event match, runtime, actual video-stream resolution, embedded graphics/occlusion, provenance/independence, and reuse rights have not been checked. The characterization is not verified evidence.</t>
         </is>
       </c>
-      <c r="AN15" s="2" t="n"/>
+      <c r="AP15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr"/>
@@ -4985,21 +5025,13 @@
       </c>
       <c r="R16" s="2" t="inlineStr"/>
       <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr">
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_and_time_match</t>
         </is>
       </c>
-      <c r="U16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="V16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="W16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -5032,56 +5064,66 @@
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AD16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
           <t>pending_verified_position</t>
         </is>
       </c>
-      <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr">
+      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AG16" s="2" t="inlineStr">
         <is>
           <t>not_assessed</t>
         </is>
       </c>
-      <c r="AF16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="AH16" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AI16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AJ16" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="AI16" s="2" t="inlineStr">
+      <c r="AK16" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ16" s="2" t="inlineStr">
+      <c r="AL16" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK16" s="2" t="inlineStr">
+      <c r="AM16" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL16" s="2" t="inlineStr">
+      <c r="AN16" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_angle_and_lineage_confirmation</t>
         </is>
       </c>
-      <c r="AM16" s="2" t="inlineStr">
+      <c r="AO16" s="2" t="inlineStr">
         <is>
           <t>User reports a long runtime may include station/signal idents or repeated static scenes, with a logo and banner obscuring the picture. These observations are not independently verified. Assess runtime and repetition separately; do not rank by duration alone. Confirm exact event and time before comparing with rQlpuY2tj-4; do not assume the same event or a different camera angle. Actual stream resolution, source credibility, independent camera status, lineage, graphics, and reuse rights remain unverified.</t>
         </is>
       </c>
-      <c r="AN16" s="2" t="n"/>
+      <c r="AP16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr"/>
@@ -5158,26 +5200,18 @@
       <c r="R17" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="S17" s="2" t="inlineStr">
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
         <is>
           <t>用户认为特色是由不同角度；是否为独立摄像机位尚未核实。</t>
         </is>
       </c>
-      <c r="T17" s="2" t="inlineStr">
+      <c r="V17" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_and_time_match</t>
         </is>
       </c>
-      <c r="U17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="W17" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -5210,59 +5244,251 @@
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AD17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
           <t>pending_verified_position</t>
         </is>
       </c>
-      <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr">
+      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AG17" s="2" t="inlineStr">
         <is>
           <t>not_assessed</t>
         </is>
       </c>
-      <c r="AF17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="AH17" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AI17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AJ17" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="AI17" s="2" t="inlineStr">
+      <c r="AK17" s="2" t="inlineStr">
         <is>
           <t>pending_direct_frame_review</t>
         </is>
       </c>
-      <c r="AJ17" s="2" t="inlineStr">
+      <c r="AL17" s="2" t="inlineStr">
         <is>
           <t>pending_source_review</t>
         </is>
       </c>
-      <c r="AK17" s="2" t="inlineStr">
+      <c r="AM17" s="2" t="inlineStr">
         <is>
           <t>pending_source_lineage_review</t>
         </is>
       </c>
-      <c r="AL17" s="2" t="inlineStr">
+      <c r="AN17" s="2" t="inlineStr">
         <is>
           <t>pending_exact_event_match_people_stage_background_audio_continuity_and_source_lineage_review</t>
         </is>
       </c>
-      <c r="AM17" s="2" t="inlineStr">
+      <c r="AO17" s="2" t="inlineStr">
         <is>
           <t>User characterizes the source as a long-form version similar to the White House official and reports a large banner and different angles. These are unverified user observations, not established event match, camera independence, or source lineage. Confirm exact event/time, people, stage/background, audio continuity, views, and repost/source lineage before comparing with rQlpuY2tj-4 or UgIivPOerNc. Duration, actual resolution, credibility, graphics, lineage, and reuse rights remain unverified. The user's overall and feature scores are subjective; the remaining rubric components and scale are unspecified.</t>
         </is>
       </c>
-      <c r="AN17" s="2" t="n"/>
+      <c r="AP17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned video lead (event match pending)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned lead only; do not compare or substitute until the exact event and time are independently matched. Do not mix with the October 13 Katie event absent that match.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>not reviewed</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>User-provided YouTube source lead (title not reviewed)</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=h30qlVplAsE</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_provenance_review</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>此链接比官方还短 还有logo 30分,但是也可以作为背景 参考 剋有看看有没有不同角度 不同花絮,作为备选片子</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>user_proposed_background_reference_and_backup_candidate_only; not approved for production</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>After exact-event/time match, look for same-event genuinely different camera angles and backstage/b-roll, verify camera/source lineage against reposts, and keep results as backup candidates until event, picture/resolution, and reuse-rights gates pass.</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AD18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>pending_verified_position</t>
+        </is>
+      </c>
+      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AG18" s="2" t="inlineStr">
+        <is>
+          <t>not_assessed</t>
+        </is>
+      </c>
+      <c r="AH18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AI18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AJ18" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AK18" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AL18" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AM18" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AN18" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_match_then_camera_angle_backstage_broll_and_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AO18" s="2" t="inlineStr">
+        <is>
+          <t>The user reports this candidate is shorter than the official source and has a logo; these observations require verification against page/runtime and actual frames. The user proposes it only as background reference/backup and requests a search for same-event alternate angles or backstage/b-roll. Do not associate it with an event from title/topic alone. Verify exact event/time, content, actual stream resolution, graphics, credibility, independent-camera status, and source/repost lineage separately. Do not select for production until event match, picture/resolution, and reuse-rights gates pass.</t>
+        </is>
+      </c>
+      <c r="AP18" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN17"/>
+  <autoFilter ref="A1:AP18"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -5280,6 +5506,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Rose Garden production status
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/event-source-review.xlsx
+++ b/outputs/event-source-review.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Directory'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$BW$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate Review'!$A$1:$BW$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'User Instructions'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Search Coverage'!$A$1:$J$4</definedName>
   </definedNames>
@@ -2214,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW54"/>
+  <dimension ref="A1:BW55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7102,20 +7102,22 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Unassigned discovery</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>social</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>2</v>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Slots 1-10</t>
+          <t>Event/category ranking pending</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -7125,23 +7127,27 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Unassigned lead only; exact event and time require independent match.</t>
+          <t>Unassigned source lead only. Do not assign an event ID or infer event date/timezone from the page title; exact event identity and content match remain unverified.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>10 News Australia on Instagram</t>
+          <t>The White House</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>@10newsau</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr"/>
+          <t>President Trump Participates in a Rose Garden Lunch, Oct. 15, 2026</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IySF_8OArvw</t>
+        </is>
+      </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact post/event/time pending</t>
+          <t>official_video_page_title_and_date_claim; exact event/content/time match unverified</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -7182,9 +7188,7 @@
       <c r="AA27" s="2" t="inlineStr"/>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
-      <c r="AD27" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD27" s="2" t="inlineStr"/>
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr"/>
       <c r="AG27" s="2" t="inlineStr">
@@ -7280,7 +7284,7 @@
       </c>
       <c r="AZ27" s="2" t="inlineStr">
         <is>
-          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
+          <t>M2 read-only checks: the official White House YouTube watch page https://www.youtube.com/watch?v=IySF_8OArvw, its oEmbed metadata https://www.youtube.com/oembed?url=https%3A%2F%2Fwww.youtube.com%2Fwatch%3Fv%3DIySF_8OArvw&amp;format=json, and the direct White House video page https://www.whitehouse.gov/videos/president-trump-participates-in-a-rose-garden-lunch-oct-15-2026/ identify The White House and the title/date claim “President Trump Participates in a Rose Garden Lunch, Oct. 15, 2026.” They do not establish direct-frame/audio content match, exact event time, or timezone; M2 did not inspect the video frames/audio. The GitHub source-intake release https://github.com/gdelt0003/gdelt0003/releases/tag/untagged-541c00d4dfd9d66e1aa8 contains asset RoseGardenLunch-IySF_8OArvw.mp4, SHA-256 e0b04fb669fd0d09f1492de6a3160bb3b6dae2e3e396be77372f4b5635da5f73; source run 38868029978 downloaded and hash-verified that release asset, not the YouTube stream itself. No acquisition record links the YouTube source to the intake asset, so source lineage is unverified. The run passed the workflow's HTTPS URL and checkbox gates with the generic White House copyright page and the direct event page; its time/timezone and lineage evidence inputs were blank. The generic policy page and operator confirmation do not establish source-specific reuse rights or independently prove exact event/source match. User processing/publication authorization = confirmed, a separate fact from these source-evidence gaps. The user permits a still BBox estimate for a review-draft lower-third mask only, labeled unverified_still_estimate; source timecode/provenance=not_verified; production_bbox_input=false/pending. It is not production-verified, and independent reviewer signature is not a user-imposed hard condition for that draft. Historical run 38832525536 published a prior layout while independent reviews were pending; it is not evidence of a current successful artifact. Current status (2026-10-16): PR #50 merged as head 690c5b0 and merge commit 4613166; all six frontend, Python, and fixture-probe CI checks passed. Current main is 775c90e8. Production run 38868029978 used main SHA c6f3931: run authorization and pinned-input validation, download of the GitHub source-intake asset (SHA-256 e0b04fb669fd0d09f1492de6a3160bb3b6dae2e3e396be77372f4b5635da5f73), and model dependency setup succeeded; transcription and translation reached 353 cues, then render failed on English cue 15 at 180.030s because it cannot fit within two lines / 68% safe width. Audit, finalization, artifact upload, and Pages deployment were skipped. Existing review release MP4 digest sha256:d51fd72a7e86fb57d8ce0521593d2b8be29aa526e3938078a2c9c6b599f69cc5, updated 2026-10-16 02:00Z, is not output of this failed run. Private artifact-only run 38895767927 on current main 775c90e8 started 11:44Z; validation, source download, and dependencies passed, render was in progress and artifact upload pending at last read. No result/artifact is yet verified for that run. Processing-evidence caveat: current validator requires HTTPS event-identity, exact-match, and rights URLs plus operator confirmation, but does not require the event-time/timezone or source-lineage URLs; run 38868029978 logged both as empty and still passed validation. Its rights URL was the general https://www.whitehouse.gov/copyright/ page, not verified source-specific reuse evidence. The current dispatch therefore records attestations, not proof that missing event/source facts or rights were established. User processing/public-review authorization remains confirmed; specific reuse rights, exact content/time match, and YouTube-to-intake lineage remain unverified. The user still estimate remains permitted only for a review draft labeled unverified_still_estimate, source timecode/provenance=not_verified, production_bbox_input=false/pending; no reviewer signature is required for that draft. No new successful artifact or production release is verified; production remains incomplete.</t>
         </is>
       </c>
       <c r="BA27" s="2" t="inlineStr"/>
@@ -7311,16 +7315,16 @@
       <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>social</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -7339,18 +7343,18 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Advocate.com</t>
+          <t>10 News Australia on Instagram</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>New White House Press Secretary Katie Zacharia claims to have passed bar in China</t>
+          <t>@10newsau</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; exact post/event/time pending</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -7391,7 +7395,9 @@
       <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr"/>
-      <c r="AD28" s="2" t="inlineStr"/>
+      <c r="AD28" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE28" s="2" t="inlineStr"/>
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="inlineStr">
@@ -7487,7 +7493,7 @@
       </c>
       <c r="AZ28" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Supplied headline is retained as source title, not endorsed as a factual description. Direct article URL and content not reviewed.</t>
+          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
         </is>
       </c>
       <c r="BA28" s="2" t="inlineStr"/>
@@ -7518,16 +7524,16 @@
       <c r="A29" s="2" t="inlineStr"/>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -7546,18 +7552,18 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Al Jazeera</t>
+          <t>Advocate.com</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>New White House press secretary Katie Zacharia holds first…</t>
+          <t>New White House Press Secretary Katie Zacharia claims to have passed bar in China</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -7594,17 +7600,11 @@
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
       <c r="Y29" s="2" t="inlineStr"/>
-      <c r="Z29" s="2" t="inlineStr">
-        <is>
-          <t>1:20</t>
-        </is>
-      </c>
+      <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="inlineStr"/>
-      <c r="AD29" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr"/>
       <c r="AG29" s="2" t="inlineStr">
@@ -7700,7 +7700,7 @@
       </c>
       <c r="AZ29" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
+          <t>Google News search result supplied by user. Supplied headline is retained as source title, not endorsed as a factual description. Direct article URL and content not reviewed.</t>
         </is>
       </c>
       <c r="BA29" s="2" t="inlineStr"/>
@@ -7731,16 +7731,16 @@
       <c r="A30" s="2" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -7764,13 +7764,13 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>White House spokesperson Katie Zacharia’s law career faces scrutiny</t>
+          <t>New White House press secretary Katie Zacharia holds first…</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -7807,11 +7807,17 @@
       <c r="W30" s="2" t="inlineStr"/>
       <c r="X30" s="2" t="inlineStr"/>
       <c r="Y30" s="2" t="inlineStr"/>
-      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>1:20</t>
+        </is>
+      </c>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
-      <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr">
@@ -7907,7 +7913,7 @@
       </c>
       <c r="AZ30" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
         </is>
       </c>
       <c r="BA30" s="2" t="inlineStr"/>
@@ -7938,16 +7944,16 @@
       <c r="A31" s="2" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
@@ -7966,18 +7972,18 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Al Jazeera English on Instagram</t>
+          <t>Al Jazeera</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>@aljazeeraenglish</t>
+          <t>White House spokesperson Katie Zacharia’s law career faces scrutiny</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact post/event/time pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -8018,9 +8024,7 @@
       <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD31" s="2" t="inlineStr"/>
       <c r="AE31" s="2" t="inlineStr"/>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr">
@@ -8116,7 +8120,7 @@
       </c>
       <c r="AZ31" s="2" t="inlineStr">
         <is>
-          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
+          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
         </is>
       </c>
       <c r="BA31" s="2" t="inlineStr"/>
@@ -8147,12 +8151,12 @@
       <c r="A32" s="2" t="inlineStr"/>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>social</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
@@ -8175,18 +8179,18 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>AP News</t>
+          <t>Al Jazeera English on Instagram</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Katie Zacharia's debut shows the pitfalls and possibilities of White House press secretary's role</t>
+          <t>@aljazeeraenglish</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; exact post/event/time pending</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -8227,7 +8231,9 @@
       <c r="AA32" s="2" t="inlineStr"/>
       <c r="AB32" s="2" t="inlineStr"/>
       <c r="AC32" s="2" t="inlineStr"/>
-      <c r="AD32" s="2" t="inlineStr"/>
+      <c r="AD32" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE32" s="2" t="inlineStr"/>
       <c r="AF32" s="2" t="inlineStr"/>
       <c r="AG32" s="2" t="inlineStr">
@@ -8323,7 +8329,7 @@
       </c>
       <c r="AZ32" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
+          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
         </is>
       </c>
       <c r="BA32" s="2" t="inlineStr"/>
@@ -8354,16 +8360,16 @@
       <c r="A33" s="2" t="inlineStr"/>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
@@ -8382,18 +8388,18 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>AP News on Instagram</t>
+          <t>AP News</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>@apnews</t>
+          <t>Katie Zacharia's debut shows the pitfalls and possibilities of White House press secretary's role</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact post/event/time pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -8434,9 +8440,7 @@
       <c r="AA33" s="2" t="inlineStr"/>
       <c r="AB33" s="2" t="inlineStr"/>
       <c r="AC33" s="2" t="inlineStr"/>
-      <c r="AD33" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD33" s="2" t="inlineStr"/>
       <c r="AE33" s="2" t="inlineStr"/>
       <c r="AF33" s="2" t="inlineStr"/>
       <c r="AG33" s="2" t="inlineStr">
@@ -8532,7 +8536,7 @@
       </c>
       <c r="AZ33" s="2" t="inlineStr">
         <is>
-          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
+          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
         </is>
       </c>
       <c r="BA33" s="2" t="inlineStr"/>
@@ -8563,16 +8567,16 @@
       <c r="A34" s="2" t="inlineStr"/>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>social</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
@@ -8591,18 +8595,18 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>AP News on Instagram</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>New White House press secretary stumbles in first briefing</t>
+          <t>@apnews</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>search_snippet_only; exact post/event/time pending</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -8639,11 +8643,7 @@
       <c r="W34" s="2" t="inlineStr"/>
       <c r="X34" s="2" t="inlineStr"/>
       <c r="Y34" s="2" t="inlineStr"/>
-      <c r="Z34" s="2" t="inlineStr">
-        <is>
-          <t>4:01</t>
-        </is>
-      </c>
+      <c r="Z34" s="2" t="inlineStr"/>
       <c r="AA34" s="2" t="inlineStr"/>
       <c r="AB34" s="2" t="inlineStr"/>
       <c r="AC34" s="2" t="inlineStr"/>
@@ -8745,7 +8745,7 @@
       </c>
       <c r="AZ34" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
+          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
         </is>
       </c>
       <c r="BA34" s="2" t="inlineStr"/>
@@ -8776,16 +8776,16 @@
       <c r="A35" s="2" t="inlineStr"/>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
@@ -8804,18 +8804,18 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>CNN</t>
+          <t>CBC</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>White House officials question how long Katie Zacharia can last after ‘brutal’ press briefing</t>
+          <t>New White House press secretary stumbles in first briefing</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -8852,11 +8852,17 @@
       <c r="W35" s="2" t="inlineStr"/>
       <c r="X35" s="2" t="inlineStr"/>
       <c r="Y35" s="2" t="inlineStr"/>
-      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>4:01</t>
+        </is>
+      </c>
       <c r="AA35" s="2" t="inlineStr"/>
       <c r="AB35" s="2" t="inlineStr"/>
       <c r="AC35" s="2" t="inlineStr"/>
-      <c r="AD35" s="2" t="inlineStr"/>
+      <c r="AD35" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE35" s="2" t="inlineStr"/>
       <c r="AF35" s="2" t="inlineStr"/>
       <c r="AG35" s="2" t="inlineStr">
@@ -8952,7 +8958,7 @@
       </c>
       <c r="AZ35" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
         </is>
       </c>
       <c r="BA35" s="2" t="inlineStr"/>
@@ -8983,16 +8989,16 @@
       <c r="A36" s="2" t="inlineStr"/>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -9011,18 +9017,18 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>FOX 29 Philadelphia</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>FULL White House Press Briefing: October 13, 2026</t>
+          <t>White House officials question how long Katie Zacharia can last after ‘brutal’ press briefing</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -9059,17 +9065,11 @@
       <c r="W36" s="2" t="inlineStr"/>
       <c r="X36" s="2" t="inlineStr"/>
       <c r="Y36" s="2" t="inlineStr"/>
-      <c r="Z36" s="2" t="inlineStr">
-        <is>
-          <t>14:34</t>
-        </is>
-      </c>
+      <c r="Z36" s="2" t="inlineStr"/>
       <c r="AA36" s="2" t="inlineStr"/>
       <c r="AB36" s="2" t="inlineStr"/>
       <c r="AC36" s="2" t="inlineStr"/>
-      <c r="AD36" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD36" s="2" t="inlineStr"/>
       <c r="AE36" s="2" t="inlineStr"/>
       <c r="AF36" s="2" t="inlineStr"/>
       <c r="AG36" s="2" t="inlineStr">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="AZ36" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
+          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
         </is>
       </c>
       <c r="BA36" s="2" t="inlineStr"/>
@@ -9196,16 +9196,16 @@
       <c r="A37" s="2" t="inlineStr"/>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -9224,18 +9224,18 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Instagram account @kenny_holston</t>
+          <t>FOX 29 Philadelphia</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>@kenny_holston</t>
+          <t>FULL White House Press Briefing: October 13, 2026</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact post/event/time pending</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -9272,7 +9272,11 @@
       <c r="W37" s="2" t="inlineStr"/>
       <c r="X37" s="2" t="inlineStr"/>
       <c r="Y37" s="2" t="inlineStr"/>
-      <c r="Z37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
       <c r="AA37" s="2" t="inlineStr"/>
       <c r="AB37" s="2" t="inlineStr"/>
       <c r="AC37" s="2" t="inlineStr"/>
@@ -9374,7 +9378,7 @@
       </c>
       <c r="AZ37" s="2" t="inlineStr">
         <is>
-          <t>User notes the handle appears to be a photographer/White House photographer account. This is not verified and does not establish that the account posted or filmed this event. Do not attribute photography or footage absent direct post inspection and reliable evidence.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
         </is>
       </c>
       <c r="BA37" s="2" t="inlineStr"/>
@@ -9414,7 +9418,7 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -9433,12 +9437,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Instagram account @thecorum</t>
+          <t>Instagram account @kenny_holston</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>@thecorum</t>
+          <t>@kenny_holston</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -9583,7 +9587,7 @@
       </c>
       <c r="AZ38" s="2" t="inlineStr">
         <is>
-          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
+          <t>User notes the handle appears to be a photographer/White House photographer account. This is not verified and does not establish that the account posted or filmed this event. Do not attribute photography or footage absent direct post inspection and reliable evidence.</t>
         </is>
       </c>
       <c r="BA38" s="2" t="inlineStr"/>
@@ -9623,7 +9627,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
@@ -9642,12 +9646,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Instagram account @valleyviewssfv</t>
+          <t>Instagram account @thecorum</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>@valleyviewssfv</t>
+          <t>@thecorum</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -9823,16 +9827,16 @@
       <c r="A40" s="2" t="inlineStr"/>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>social</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
@@ -9851,18 +9855,18 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>MS NOW</t>
+          <t>Instagram account @valleyviewssfv</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Not ready for primetime: New press secretary stumbles in her debut</t>
+          <t>@valleyviewssfv</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; exact post/event/time pending</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -9903,7 +9907,9 @@
       <c r="AA40" s="2" t="inlineStr"/>
       <c r="AB40" s="2" t="inlineStr"/>
       <c r="AC40" s="2" t="inlineStr"/>
-      <c r="AD40" s="2" t="inlineStr"/>
+      <c r="AD40" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE40" s="2" t="inlineStr"/>
       <c r="AF40" s="2" t="inlineStr"/>
       <c r="AG40" s="2" t="inlineStr">
@@ -9999,7 +10005,7 @@
       </c>
       <c r="AZ40" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
+          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
         </is>
       </c>
       <c r="BA40" s="2" t="inlineStr"/>
@@ -10030,16 +10036,16 @@
       <c r="A41" s="2" t="inlineStr"/>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -10058,18 +10064,18 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>MS NOW on Instagram</t>
+          <t>MS NOW</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>@msnownews</t>
+          <t>Not ready for primetime: New press secretary stumbles in her debut</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact post/event/time pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -10110,9 +10116,7 @@
       <c r="AA41" s="2" t="inlineStr"/>
       <c r="AB41" s="2" t="inlineStr"/>
       <c r="AC41" s="2" t="inlineStr"/>
-      <c r="AD41" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD41" s="2" t="inlineStr"/>
       <c r="AE41" s="2" t="inlineStr"/>
       <c r="AF41" s="2" t="inlineStr"/>
       <c r="AG41" s="2" t="inlineStr">
@@ -10208,7 +10212,7 @@
       </c>
       <c r="AZ41" s="2" t="inlineStr">
         <is>
-          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
+          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
         </is>
       </c>
       <c r="BA41" s="2" t="inlineStr"/>
@@ -10239,16 +10243,16 @@
       <c r="A42" s="2" t="inlineStr"/>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>social</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
@@ -10267,18 +10271,18 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NBC News</t>
+          <t>MS NOW on Instagram</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Katie Zacharia holds first White House press briefing weeks…</t>
+          <t>@msnownews</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>search_snippet_only; exact post/event/time pending</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -10315,11 +10319,7 @@
       <c r="W42" s="2" t="inlineStr"/>
       <c r="X42" s="2" t="inlineStr"/>
       <c r="Y42" s="2" t="inlineStr"/>
-      <c r="Z42" s="2" t="inlineStr">
-        <is>
-          <t>3:17</t>
-        </is>
-      </c>
+      <c r="Z42" s="2" t="inlineStr"/>
       <c r="AA42" s="2" t="inlineStr"/>
       <c r="AB42" s="2" t="inlineStr"/>
       <c r="AC42" s="2" t="inlineStr"/>
@@ -10421,7 +10421,7 @@
       </c>
       <c r="AZ42" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
+          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
         </is>
       </c>
       <c r="BA42" s="2" t="inlineStr"/>
@@ -10452,16 +10452,16 @@
       <c r="A43" s="2" t="inlineStr"/>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
@@ -10480,18 +10480,18 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>PBS</t>
+          <t>NBC News</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>WATCH: New White House press secretary Katie Zacharia takes few questions in short first briefing</t>
+          <t>Katie Zacharia holds first White House press briefing weeks…</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -10528,11 +10528,17 @@
       <c r="W43" s="2" t="inlineStr"/>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
-      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>3:17</t>
+        </is>
+      </c>
       <c r="AA43" s="2" t="inlineStr"/>
       <c r="AB43" s="2" t="inlineStr"/>
       <c r="AC43" s="2" t="inlineStr"/>
-      <c r="AD43" s="2" t="inlineStr"/>
+      <c r="AD43" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE43" s="2" t="inlineStr"/>
       <c r="AF43" s="2" t="inlineStr"/>
       <c r="AG43" s="2" t="inlineStr">
@@ -10628,7 +10634,7 @@
       </c>
       <c r="AZ43" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. The title suggests a video/report but does not establish direct event footage, exact event/time, or camera source. Direct article URL and content not reviewed.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
         </is>
       </c>
       <c r="BA43" s="2" t="inlineStr"/>
@@ -10659,16 +10665,16 @@
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
@@ -10687,18 +10693,18 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Reuters</t>
+          <t>PBS</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>LIVE: New White House press secretary Katie Zacharia holds…</t>
+          <t>WATCH: New White House press secretary Katie Zacharia takes few questions in short first briefing</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -10739,9 +10745,7 @@
       <c r="AA44" s="2" t="inlineStr"/>
       <c r="AB44" s="2" t="inlineStr"/>
       <c r="AC44" s="2" t="inlineStr"/>
-      <c r="AD44" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD44" s="2" t="inlineStr"/>
       <c r="AE44" s="2" t="inlineStr"/>
       <c r="AF44" s="2" t="inlineStr"/>
       <c r="AG44" s="2" t="inlineStr">
@@ -10837,7 +10841,7 @@
       </c>
       <c r="AZ44" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Page content, exact event/time, runtime, camera angle, lineage, and rights remain unverified.</t>
+          <t>Google News search result supplied by user. The title suggests a video/report but does not establish direct event footage, exact event/time, or camera source. Direct article URL and content not reviewed.</t>
         </is>
       </c>
       <c r="BA44" s="2" t="inlineStr"/>
@@ -10868,16 +10872,16 @@
       <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
@@ -10901,13 +10905,13 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>New White House press secretary Katie Zacharia's legal career draws scrutiny</t>
+          <t>LIVE: New White House press secretary Katie Zacharia holds…</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -10947,12 +10951,10 @@
       <c r="Z45" s="2" t="inlineStr"/>
       <c r="AA45" s="2" t="inlineStr"/>
       <c r="AB45" s="2" t="inlineStr"/>
-      <c r="AC45" s="2" t="inlineStr">
-        <is>
-          <t>Oct 14 (user-reported snippet metadata; not event time)</t>
-        </is>
-      </c>
-      <c r="AD45" s="2" t="inlineStr"/>
+      <c r="AC45" s="2" t="inlineStr"/>
+      <c r="AD45" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE45" s="2" t="inlineStr"/>
       <c r="AF45" s="2" t="inlineStr"/>
       <c r="AG45" s="2" t="inlineStr">
@@ -11048,7 +11050,7 @@
       </c>
       <c r="AZ45" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Title/topic, publication metadata, and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Page content, exact event/time, runtime, camera angle, lineage, and rights remain unverified.</t>
         </is>
       </c>
       <c r="BA45" s="2" t="inlineStr"/>
@@ -11079,16 +11081,16 @@
       <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
@@ -11107,18 +11109,18 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Right Side Broadcasting Network</t>
+          <t>Reuters</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Katie Zacharia Holds First Press Briefing…</t>
+          <t>New White House press secretary Katie Zacharia's legal career draws scrutiny</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -11155,17 +11157,15 @@
       <c r="W46" s="2" t="inlineStr"/>
       <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="2" t="inlineStr"/>
-      <c r="Z46" s="2" t="inlineStr">
-        <is>
-          <t>14:08</t>
-        </is>
-      </c>
+      <c r="Z46" s="2" t="inlineStr"/>
       <c r="AA46" s="2" t="inlineStr"/>
       <c r="AB46" s="2" t="inlineStr"/>
-      <c r="AC46" s="2" t="inlineStr"/>
-      <c r="AD46" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AC46" s="2" t="inlineStr">
+        <is>
+          <t>Oct 14 (user-reported snippet metadata; not event time)</t>
+        </is>
+      </c>
+      <c r="AD46" s="2" t="inlineStr"/>
       <c r="AE46" s="2" t="inlineStr"/>
       <c r="AF46" s="2" t="inlineStr"/>
       <c r="AG46" s="2" t="inlineStr">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="AZ46" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
+          <t>Google News search result supplied by user. Title/topic, publication metadata, and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
         </is>
       </c>
       <c r="BA46" s="2" t="inlineStr"/>
@@ -11292,12 +11292,12 @@
       <c r="A47" s="2" t="inlineStr"/>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
@@ -11320,18 +11320,18 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Right Side Broadcasting Network on Facebook</t>
+          <t>Right Side Broadcasting Network</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Right Side Broadcasting Network Facebook search-result post</t>
+          <t>Katie Zacharia Holds First Press Briefing…</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact page/event/time pending</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -11368,7 +11368,11 @@
       <c r="W47" s="2" t="inlineStr"/>
       <c r="X47" s="2" t="inlineStr"/>
       <c r="Y47" s="2" t="inlineStr"/>
-      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
       <c r="AA47" s="2" t="inlineStr"/>
       <c r="AB47" s="2" t="inlineStr"/>
       <c r="AC47" s="2" t="inlineStr"/>
@@ -11470,7 +11474,7 @@
       </c>
       <c r="AZ47" s="2" t="inlineStr">
         <is>
-          <t>User-reported Google social-platform search result; no direct post URL supplied. No post content, event match, camera source, or lineage verified.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
         </is>
       </c>
       <c r="BA47" s="2" t="inlineStr"/>
@@ -11501,16 +11505,16 @@
       <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>social</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
@@ -11529,18 +11533,18 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Sinar Daily</t>
+          <t>Right Side Broadcasting Network on Facebook</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Trump's new press secretary Katie Zacharia faces scrutiny over credentials</t>
+          <t>Right Side Broadcasting Network Facebook search-result post</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of direct event footage</t>
+          <t>search_snippet_only; exact page/event/time pending</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -11581,7 +11585,9 @@
       <c r="AA48" s="2" t="inlineStr"/>
       <c r="AB48" s="2" t="inlineStr"/>
       <c r="AC48" s="2" t="inlineStr"/>
-      <c r="AD48" s="2" t="inlineStr"/>
+      <c r="AD48" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE48" s="2" t="inlineStr"/>
       <c r="AF48" s="2" t="inlineStr"/>
       <c r="AG48" s="2" t="inlineStr">
@@ -11677,7 +11683,7 @@
       </c>
       <c r="AZ48" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
+          <t>User-reported Google social-platform search result; no direct post URL supplied. No post content, event match, camera source, or lineage verified.</t>
         </is>
       </c>
       <c r="BA48" s="2" t="inlineStr"/>
@@ -11717,7 +11723,7 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
@@ -11736,12 +11742,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>The Guardian</t>
+          <t>Sinar Daily</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Enter the Zachbot: Trump’s new press secretary malfunctions on podium debut</t>
+          <t>Trump's new press secretary Katie Zacharia faces scrutiny over credentials</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
@@ -11884,7 +11890,7 @@
       </c>
       <c r="AZ49" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. Supplied headline is retained as source title, not endorsed as a factual description. Direct article URL and content not reviewed.</t>
+          <t>Google News search result supplied by user. Title/topic and any claims remain unverified; this is a reporting lead, not direct footage or proof of event facts. Direct article URL not supplied.</t>
         </is>
       </c>
       <c r="BA49" s="2" t="inlineStr"/>
@@ -11915,16 +11921,16 @@
       <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
@@ -11943,18 +11949,18 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>The Guardian</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>The New White House Press Secretary Has Awkward Debut</t>
+          <t>Enter the Zachbot: Trump’s new press secretary malfunctions on podium debut</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>news_search_lead; not evidence of direct event footage</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -11991,17 +11997,11 @@
       <c r="W50" s="2" t="inlineStr"/>
       <c r="X50" s="2" t="inlineStr"/>
       <c r="Y50" s="2" t="inlineStr"/>
-      <c r="Z50" s="2" t="inlineStr">
-        <is>
-          <t>0:53</t>
-        </is>
-      </c>
+      <c r="Z50" s="2" t="inlineStr"/>
       <c r="AA50" s="2" t="inlineStr"/>
       <c r="AB50" s="2" t="inlineStr"/>
       <c r="AC50" s="2" t="inlineStr"/>
-      <c r="AD50" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD50" s="2" t="inlineStr"/>
       <c r="AE50" s="2" t="inlineStr"/>
       <c r="AF50" s="2" t="inlineStr"/>
       <c r="AG50" s="2" t="inlineStr">
@@ -12097,7 +12097,7 @@
       </c>
       <c r="AZ50" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
+          <t>Google News search result supplied by user. Supplied headline is retained as source title, not endorsed as a factual description. Direct article URL and content not reviewed.</t>
         </is>
       </c>
       <c r="BA50" s="2" t="inlineStr"/>
@@ -12128,12 +12128,12 @@
       <c r="A51" s="2" t="inlineStr"/>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>video</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
@@ -12156,18 +12156,18 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>The White House</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Katie Zacharia Delivers Powerful Inaugural Briefing…</t>
+          <t>The New White House Press Secretary Has Awkward Debut</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>news_search_lead; not evidence of independent reporting</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -12204,11 +12204,17 @@
       <c r="W51" s="2" t="inlineStr"/>
       <c r="X51" s="2" t="inlineStr"/>
       <c r="Y51" s="2" t="inlineStr"/>
-      <c r="Z51" s="2" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
+          <t>0:53</t>
+        </is>
+      </c>
       <c r="AA51" s="2" t="inlineStr"/>
       <c r="AB51" s="2" t="inlineStr"/>
       <c r="AC51" s="2" t="inlineStr"/>
-      <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AD51" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE51" s="2" t="inlineStr"/>
       <c r="AF51" s="2" t="inlineStr"/>
       <c r="AG51" s="2" t="inlineStr">
@@ -12304,7 +12310,7 @@
       </c>
       <c r="AZ51" s="2" t="inlineStr">
         <is>
-          <t>Google News search result supplied by user. The supplied title appears to use official promotional framing; this is not treated as a neutral claim or verified fact. Direct page URL and content not reviewed.</t>
+          <t>Google video search snippet supplied by user; direct result URL not supplied. Snippet runtime is metadata only, not measured. Not proof of exact event/time, source page content, or an independent camera angle.</t>
         </is>
       </c>
       <c r="BA51" s="2" t="inlineStr"/>
@@ -12335,12 +12341,12 @@
       <c r="A52" s="2" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Katie briefing social search leads (event/source match unverified)</t>
+          <t>Katie Zacharia briefing (Google News search leads; event and topic match unverified)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>news</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
@@ -12363,18 +12369,18 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Times Now on Instagram</t>
+          <t>The White House</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>@timesnow</t>
+          <t>Katie Zacharia Delivers Powerful Inaugural Briefing…</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; exact post/event/time pending</t>
+          <t>news_search_lead; not evidence of independent reporting</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -12415,9 +12421,7 @@
       <c r="AA52" s="2" t="inlineStr"/>
       <c r="AB52" s="2" t="inlineStr"/>
       <c r="AC52" s="2" t="inlineStr"/>
-      <c r="AD52" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="AD52" s="2" t="inlineStr"/>
       <c r="AE52" s="2" t="inlineStr"/>
       <c r="AF52" s="2" t="inlineStr"/>
       <c r="AG52" s="2" t="inlineStr">
@@ -12513,7 +12517,7 @@
       </c>
       <c r="AZ52" s="2" t="inlineStr">
         <is>
-          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
+          <t>Google News search result supplied by user. The supplied title appears to use official promotional framing; this is not treated as a neutral claim or verified fact. Direct page URL and content not reviewed.</t>
         </is>
       </c>
       <c r="BA52" s="2" t="inlineStr"/>
@@ -12544,7 +12548,7 @@
       <c r="A53" s="2" t="inlineStr"/>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
+          <t>Katie briefing social search leads (event/source match unverified)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -12553,7 +12557,7 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
@@ -12572,18 +12576,18 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>WFSB on Facebook</t>
+          <t>Times Now on Instagram</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>WFSB Facebook short (snippet links WFSB article)</t>
+          <t>@timesnow</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>search_snippet_only; page/event/time/camera match pending</t>
+          <t>search_snippet_only; exact post/event/time pending</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -12620,11 +12624,7 @@
       <c r="W53" s="2" t="inlineStr"/>
       <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="2" t="inlineStr"/>
-      <c r="Z53" s="2" t="inlineStr">
-        <is>
-          <t>0:22</t>
-        </is>
-      </c>
+      <c r="Z53" s="2" t="inlineStr"/>
       <c r="AA53" s="2" t="inlineStr"/>
       <c r="AB53" s="2" t="inlineStr"/>
       <c r="AC53" s="2" t="inlineStr"/>
@@ -12726,7 +12726,7 @@
       </c>
       <c r="AZ53" s="2" t="inlineStr">
         <is>
-          <t>Google video search snippet supplied by user; direct Facebook page URL not supplied. Snippet runtime is metadata only. The search snippet references a WFSB article; page contents, event/time match, camera angle, lineage, and rights are unreviewed.</t>
+          <t>User-reported account search result; account handle does not identify a specific post or establish source footage. Direct post URL, content, event match, and lineage remain unknown.</t>
         </is>
       </c>
       <c r="BA53" s="2" t="inlineStr"/>
@@ -12757,40 +12757,46 @@
       <c r="A54" s="2" t="inlineStr"/>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Unassigned screenshot/time-marker report</t>
+          <t>Oct 13 Katie briefing (search leads; event/source match unverified)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>unassigned screenshot</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+          <t>social</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Identity unresolved</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr"/>
+          <t>Slots 1-10</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>source directness, exact-event evidence, direct-URL availability, recency when known, then publisher/URL; popularity is excluded</t>
+        </is>
+      </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>No video ID or source URL supplied. Keep this display report separate from all candidate videos until the user identifies it.</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr"/>
+          <t>Unassigned lead only; exact event and time require independent match.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>WFSB on Facebook</t>
+        </is>
+      </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>User-described screenshot; source unresolved</t>
+          <t>WFSB Facebook short (snippet links WFSB article)</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>unassigned</t>
+          <t>search_snippet_only; page/event/time/camera match pending</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -12805,129 +12811,336 @@
       </c>
       <c r="N54" s="2" t="inlineStr"/>
       <c r="O54" s="2" t="inlineStr"/>
-      <c r="P54" s="2" t="inlineStr"/>
-      <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_provenance_review</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>pending_rights_review</t>
+        </is>
+      </c>
       <c r="S54" s="2" t="inlineStr"/>
       <c r="T54" s="2" t="inlineStr"/>
       <c r="U54" s="2" t="inlineStr"/>
-      <c r="V54" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="W54" s="2" t="inlineStr">
-        <is>
-          <t>Unlinked screenshot-only report; scores are not assigned to a video candidate.</t>
-        </is>
-      </c>
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
       <c r="X54" s="2" t="inlineStr"/>
-      <c r="Y54" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="Z54" s="2" t="inlineStr"/>
+      <c r="Y54" s="2" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>0:22</t>
+        </is>
+      </c>
       <c r="AA54" s="2" t="inlineStr"/>
       <c r="AB54" s="2" t="inlineStr"/>
       <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr"/>
+      <c r="AD54" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="AE54" s="2" t="inlineStr"/>
       <c r="AF54" s="2" t="inlineStr"/>
-      <c r="AG54" s="2" t="inlineStr"/>
-      <c r="AH54" s="2" t="inlineStr"/>
-      <c r="AI54" s="2" t="inlineStr"/>
-      <c r="AJ54" s="2" t="inlineStr"/>
-      <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr"/>
-      <c r="AM54" s="2" t="inlineStr"/>
-      <c r="AN54" s="2" t="inlineStr"/>
-      <c r="AO54" s="2" t="inlineStr"/>
-      <c r="AP54" s="2" t="inlineStr"/>
+      <c r="AG54" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_and_time_match</t>
+        </is>
+      </c>
+      <c r="AH54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AI54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AJ54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AK54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AL54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AM54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AN54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AO54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AP54" s="2" t="inlineStr">
+        <is>
+          <t>pending_verified_position</t>
+        </is>
+      </c>
       <c r="AQ54" s="2" t="inlineStr"/>
-      <c r="AR54" s="2" t="inlineStr"/>
-      <c r="AS54" s="2" t="inlineStr"/>
-      <c r="AT54" s="2" t="inlineStr"/>
-      <c r="AU54" s="2" t="inlineStr"/>
-      <c r="AV54" s="2" t="inlineStr"/>
-      <c r="AW54" s="2" t="inlineStr"/>
-      <c r="AX54" s="2" t="inlineStr"/>
-      <c r="AY54" s="2" t="inlineStr"/>
+      <c r="AR54" s="2" t="inlineStr">
+        <is>
+          <t>not_assessed</t>
+        </is>
+      </c>
+      <c r="AS54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AT54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AU54" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AV54" s="2" t="inlineStr">
+        <is>
+          <t>pending_direct_frame_review</t>
+        </is>
+      </c>
+      <c r="AW54" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_review</t>
+        </is>
+      </c>
+      <c r="AX54" s="2" t="inlineStr">
+        <is>
+          <t>pending_source_lineage_review</t>
+        </is>
+      </c>
+      <c r="AY54" s="2" t="inlineStr">
+        <is>
+          <t>pending_exact_event_angle_and_lineage_confirmation</t>
+        </is>
+      </c>
       <c r="AZ54" s="2" t="inlineStr">
         <is>
+          <t>Google video search snippet supplied by user; direct Facebook page URL not supplied. Snippet runtime is metadata only. The search snippet references a WFSB article; page contents, event/time match, camera angle, lineage, and rights are unreviewed.</t>
+        </is>
+      </c>
+      <c r="BA54" s="2" t="inlineStr"/>
+      <c r="BB54" s="2" t="inlineStr"/>
+      <c r="BC54" s="2" t="inlineStr"/>
+      <c r="BD54" s="2" t="inlineStr"/>
+      <c r="BE54" s="2" t="inlineStr"/>
+      <c r="BF54" s="2" t="inlineStr"/>
+      <c r="BG54" s="2" t="inlineStr"/>
+      <c r="BH54" s="2" t="inlineStr"/>
+      <c r="BI54" s="2" t="inlineStr"/>
+      <c r="BJ54" s="2" t="inlineStr"/>
+      <c r="BK54" s="2" t="inlineStr"/>
+      <c r="BL54" s="2" t="inlineStr"/>
+      <c r="BM54" s="2" t="inlineStr"/>
+      <c r="BN54" s="2" t="inlineStr"/>
+      <c r="BO54" s="2" t="inlineStr"/>
+      <c r="BP54" s="2" t="inlineStr"/>
+      <c r="BQ54" s="2" t="inlineStr"/>
+      <c r="BR54" s="2" t="inlineStr"/>
+      <c r="BS54" s="2" t="inlineStr"/>
+      <c r="BT54" s="2" t="inlineStr"/>
+      <c r="BU54" s="2" t="inlineStr"/>
+      <c r="BV54" s="2" t="inlineStr"/>
+      <c r="BW54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned screenshot/time-marker report</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>unassigned screenshot</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Identity unresolved</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>No video ID or source URL supplied. Keep this display report separate from all candidate videos until the user identifies it.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>User-described screenshot; source unresolved</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>unassigned</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr"/>
+      <c r="Q55" s="2" t="inlineStr"/>
+      <c r="R55" s="2" t="inlineStr"/>
+      <c r="S55" s="2" t="inlineStr"/>
+      <c r="T55" s="2" t="inlineStr"/>
+      <c r="U55" s="2" t="inlineStr"/>
+      <c r="V55" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="W55" s="2" t="inlineStr">
+        <is>
+          <t>Unlinked screenshot-only report; scores are not assigned to a video candidate.</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr"/>
+      <c r="Y55" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z55" s="2" t="inlineStr"/>
+      <c r="AA55" s="2" t="inlineStr"/>
+      <c r="AB55" s="2" t="inlineStr"/>
+      <c r="AC55" s="2" t="inlineStr"/>
+      <c r="AD55" s="2" t="inlineStr"/>
+      <c r="AE55" s="2" t="inlineStr"/>
+      <c r="AF55" s="2" t="inlineStr"/>
+      <c r="AG55" s="2" t="inlineStr"/>
+      <c r="AH55" s="2" t="inlineStr"/>
+      <c r="AI55" s="2" t="inlineStr"/>
+      <c r="AJ55" s="2" t="inlineStr"/>
+      <c r="AK55" s="2" t="inlineStr"/>
+      <c r="AL55" s="2" t="inlineStr"/>
+      <c r="AM55" s="2" t="inlineStr"/>
+      <c r="AN55" s="2" t="inlineStr"/>
+      <c r="AO55" s="2" t="inlineStr"/>
+      <c r="AP55" s="2" t="inlineStr"/>
+      <c r="AQ55" s="2" t="inlineStr"/>
+      <c r="AR55" s="2" t="inlineStr"/>
+      <c r="AS55" s="2" t="inlineStr"/>
+      <c r="AT55" s="2" t="inlineStr"/>
+      <c r="AU55" s="2" t="inlineStr"/>
+      <c r="AV55" s="2" t="inlineStr"/>
+      <c r="AW55" s="2" t="inlineStr"/>
+      <c r="AX55" s="2" t="inlineStr"/>
+      <c r="AY55" s="2" t="inlineStr"/>
+      <c r="AZ55" s="2" t="inlineStr">
+        <is>
           <t>The reported display does not establish marker date, timezone correctness, live status, or event time. Player chrome is not event time. No video ID was supplied; do not infer one from the displayed runtime.</t>
         </is>
       </c>
-      <c r="BA54" s="2" t="inlineStr">
+      <c r="BA55" s="2" t="inlineStr">
         <is>
           <t>user-reported; candidate unresolved</t>
         </is>
       </c>
-      <c r="BB54" s="2" t="inlineStr">
+      <c r="BB55" s="2" t="inlineStr">
         <is>
           <t>9:44 AM ET</t>
         </is>
       </c>
-      <c r="BC54" s="2" t="inlineStr">
+      <c r="BC55" s="2" t="inlineStr">
         <is>
           <t>lower-left channel/logo zone (user-described)</t>
         </is>
       </c>
-      <c r="BD54" s="2" t="n"/>
-      <c r="BE54" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="BF54" s="2" t="inlineStr">
+      <c r="BD55" s="2" t="n"/>
+      <c r="BE55" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BF55" s="2" t="inlineStr">
         <is>
           <t>ET (as displayed; correctness unverified)</t>
         </is>
       </c>
-      <c r="BG54" s="2" t="n"/>
-      <c r="BH54" s="2" t="n"/>
-      <c r="BI54" s="2" t="inlineStr">
+      <c r="BG55" s="2" t="n"/>
+      <c r="BH55" s="2" t="n"/>
+      <c r="BI55" s="2" t="inlineStr">
         <is>
           <t>user-described screenshot appearance only; screenshot artifact and candidate identity unresolved</t>
         </is>
       </c>
-      <c r="BJ54" s="2" t="inlineStr">
+      <c r="BJ55" s="2" t="inlineStr">
         <is>
           <t>0:10 / 14:07</t>
         </is>
       </c>
-      <c r="BK54" s="2" t="n"/>
-      <c r="BL54" s="2" t="n"/>
-      <c r="BM54" s="2" t="n"/>
-      <c r="BN54" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="BO54" s="2" t="n"/>
-      <c r="BP54" s="2" t="n"/>
-      <c r="BQ54" s="2" t="n"/>
-      <c r="BR54" s="2" t="n"/>
-      <c r="BS54" s="2" t="inlineStr">
+      <c r="BK55" s="2" t="n"/>
+      <c r="BL55" s="2" t="n"/>
+      <c r="BM55" s="2" t="n"/>
+      <c r="BN55" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BO55" s="2" t="n"/>
+      <c r="BP55" s="2" t="n"/>
+      <c r="BQ55" s="2" t="n"/>
+      <c r="BR55" s="2" t="n"/>
+      <c r="BS55" s="2" t="inlineStr">
         <is>
           <t>not_computable_until_candidate_and_comparable_verified_event_time_are_evidenced</t>
         </is>
       </c>
-      <c r="BT54" s="2" t="inlineStr">
+      <c r="BT55" s="2" t="inlineStr">
         <is>
           <t>not_computed</t>
         </is>
       </c>
-      <c r="BU54" s="2" t="n"/>
-      <c r="BV54" s="2" t="inlineStr">
+      <c r="BU55" s="2" t="n"/>
+      <c r="BV55" s="2" t="inlineStr">
         <is>
           <t>No threshold defined.</t>
         </is>
       </c>
-      <c r="BW54" s="2" t="inlineStr">
+      <c r="BW55" s="2" t="inlineStr">
         <is>
           <t>User overall score 60 and feature score 15; unassigned and not attached to any candidate. The reported display does not establish marker date, timezone correctness, live status, or event time. Player chrome is not event time. No video ID was supplied; do not infer one from the displayed runtime.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BW54"/>
+  <autoFilter ref="A1:BW55"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
@@ -12979,6 +13192,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>